<commit_message>
Promote Master 4 to live CATS and rename 114R/115R to 120R/120L.
Archive the unused West Yard sheets, drop orphaned IH435, and refresh LCOS inventory so the rename has one aligned SoR before the next numbering pass.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
+++ b/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -732,7 +732,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C4-OU2-4</t>
+          <t>C4-OU2-5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -752,45 +752,49 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>435</t>
+          <t>436</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>IH435</t>
+          <t>IH436</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>spare C4-OU2-4</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
+          <t>101RA</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>101RA</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>SPARE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>track/signalhead/IH435</t>
+          <t>track/signalhead/IH436</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; spare (was 102LA Bottom); packed slot held so 101RA stays IH436</t>
+          <t>LCOS Signal 4 UID 36; Digicon mast '101RA'</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C4-OU2-5</t>
+          <t>C4-OU2-6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -810,27 +814,27 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>436</t>
+          <t>437</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>IH436</t>
+          <t>IH437</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>101RA</t>
+          <t>101RB</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>101RA</t>
+          <t>101RB</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -840,19 +844,19 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>track/signalhead/IH436</t>
+          <t>track/signalhead/IH437</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; Digicon mast '101RA'</t>
+          <t>LCOS Signal 5 UID 37; Digicon mast '101RB'</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C4-OU2-6</t>
+          <t>C4-OU3-1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -872,49 +876,49 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>437</t>
+          <t>438</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>IH437</t>
+          <t>IH438</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>101RB</t>
+          <t>100L Top</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>101RB</t>
+          <t>100L</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>T</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>track/signalhead/IH437</t>
+          <t>track/signalhead/IH438</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; Digicon mast '101RB'</t>
+          <t>LCOS Signal 6 UID 38; Digicon mast '100L'</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C4-OU3-1</t>
+          <t>C4-OU3-2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -934,22 +938,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>438</t>
+          <t>439</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>IH438</t>
+          <t>IH439</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>100L Top</t>
+          <t>100L Bottom</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -959,86 +963,86 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>track/signalhead/IH438</t>
+          <t>track/signalhead/IH439</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; Digicon mast '100L'</t>
+          <t>LCOS Signal 7 UID 39; Digicon mast '100L'</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C4-OU3-2</t>
+          <t>C1-OU2-1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>Helix - Lower (Barn / West Yard)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>439</t>
+          <t>1332</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>IH439</t>
+          <t>IH1332</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>100L Bottom</t>
+          <t>117RA Top</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>100L</t>
+          <t>117RA</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>track/signalhead/IH439</t>
+          <t>track/signalhead/IH1332</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; Digicon mast '100L'</t>
+          <t>LCOS Signal 0 UID 32; Digicon mast '117RA'</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C1-OU2-1</t>
+          <t>C1-OU2-2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1058,22 +1062,22 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1332</t>
+          <t>1333</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>IH1332</t>
+          <t>IH1333</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>117RA Top</t>
+          <t>117RA Bottom</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1083,24 +1087,24 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1332</t>
+          <t>track/signalhead/IH1333</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; Digicon mast '117RA'</t>
+          <t>LCOS Signal 1 UID 33; Digicon mast '117RA'</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C1-OU2-2</t>
+          <t>C1-OU2-3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1120,49 +1124,49 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1333</t>
+          <t>1334</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>IH1333</t>
+          <t>IH1334</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>117RA Bottom</t>
+          <t>117LB</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>117RA</t>
+          <t>117LB</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>S</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1333</t>
+          <t>track/signalhead/IH1334</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; Digicon mast '117RA'</t>
+          <t>LCOS Signal 2 UID 34; Digicon mast '117LB'</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C1-OU2-3</t>
+          <t>C1-OU2-4</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1182,49 +1186,49 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1334</t>
+          <t>1335</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>IH1334</t>
+          <t>IH1335</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>117LB</t>
+          <t>117RB Top</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>117LB</t>
+          <t>117RB</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>T</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1334</t>
+          <t>track/signalhead/IH1335</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; Digicon mast '117LB'</t>
+          <t>LCOS Signal 3 UID 35; Digicon mast '117RB'</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C1-OU2-4</t>
+          <t>C1-OU2-5</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1244,22 +1248,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1335</t>
+          <t>1336</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>IH1335</t>
+          <t>IH1336</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>117RB Top</t>
+          <t>117RB Bottom</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1269,24 +1273,24 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1335</t>
+          <t>track/signalhead/IH1336</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; Digicon mast '117RB'</t>
+          <t>LCOS Signal 4 UID 36; Digicon mast '117RB'</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C1-OU2-5</t>
+          <t>C1-OU2-6</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1306,49 +1310,49 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1336</t>
+          <t>1337</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>IH1336</t>
+          <t>IH1337</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>117RB Bottom</t>
+          <t>117LA Top</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>117RB</t>
+          <t>117LA</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1336</t>
+          <t>track/signalhead/IH1337</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; Digicon mast '117RB'</t>
+          <t>LCOS Signal 5 UID 37; Digicon mast '117LA'</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C1-OU2-6</t>
+          <t>C1-OU3-1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1368,22 +1372,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1337</t>
+          <t>1338</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>IH1337</t>
+          <t>IH1338</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>117LA Top</t>
+          <t>117LA Bottom</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1393,86 +1397,86 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1337</t>
+          <t>track/signalhead/IH1338</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; Digicon mast '117LA'</t>
+          <t>LCOS Signal 6 UID 38; Digicon mast '117LA'</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C1-OU3-1</t>
+          <t>C7-OU2-1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>North - Upper (East End)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1338</t>
+          <t>1232</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>IH1338</t>
+          <t>IH1232</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>117LA Bottom</t>
+          <t>111RA Top</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>117LA</t>
+          <t>111RA</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1338</t>
+          <t>track/signalhead/IH1232</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; Digicon mast '117LA'</t>
+          <t>LCOS Signal 0 UID 32; Digicon mast '111RA'</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>C7-OU2-1</t>
+          <t>C7-OU2-2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1492,22 +1496,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1232</t>
+          <t>1233</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>IH1232</t>
+          <t>IH1233</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>111RA Top</t>
+          <t>111RA Bottom</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1517,24 +1521,24 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1232</t>
+          <t>track/signalhead/IH1233</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; Digicon mast '111RA'</t>
+          <t>LCOS Signal 1 UID 33; Digicon mast '111RA'</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>C7-OU2-2</t>
+          <t>C7-OU2-3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1554,49 +1558,49 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1233</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>IH1233</t>
+          <t>IH1234</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>111RA Bottom</t>
+          <t>111L Top</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>111RA</t>
+          <t>111L</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1233</t>
+          <t>track/signalhead/IH1234</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; Digicon mast '111RA'</t>
+          <t>LCOS Signal 2 UID 34; Digicon mast '111L'</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C7-OU2-3</t>
+          <t>C7-OU2-4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1616,22 +1620,22 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1234</t>
+          <t>1235</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>IH1234</t>
+          <t>IH1235</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>111L Top</t>
+          <t>111L Bottom</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1641,24 +1645,24 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1234</t>
+          <t>track/signalhead/IH1235</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; Digicon mast '111L'</t>
+          <t>LCOS Signal 3 UID 35; Digicon mast '111L'</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>C7-OU2-4</t>
+          <t>C7-OU2-5</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1678,49 +1682,49 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1235</t>
+          <t>1236</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>IH1235</t>
+          <t>IH1236</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>111L Bottom</t>
+          <t>111RB</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>111L</t>
+          <t>111RB</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>S</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1235</t>
+          <t>track/signalhead/IH1236</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; Digicon mast '111L'</t>
+          <t>LCOS Signal 4 UID 36; Digicon mast '111RB'</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>C7-OU2-5</t>
+          <t>C7-OU2-6</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1740,49 +1744,49 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1236</t>
+          <t>1237</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>IH1236</t>
+          <t>IH1237</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>111RB</t>
+          <t>112L Top</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>111RB</t>
+          <t>112L</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>T</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1236</t>
+          <t>track/signalhead/IH1237</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; Digicon mast '111RB'</t>
+          <t>LCOS Signal 5 UID 37; Digicon mast '112L'</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>C7-OU2-6</t>
+          <t>C7-OU3-1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1802,22 +1806,22 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1237</t>
+          <t>1238</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>IH1237</t>
+          <t>IH1238</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>112L Top</t>
+          <t>112L Bottom</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1827,24 +1831,24 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1237</t>
+          <t>track/signalhead/IH1238</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; Digicon mast '112L'</t>
+          <t>LCOS Signal 6 UID 38; Digicon mast '112L'</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>C7-OU3-1</t>
+          <t>C7-OU3-2</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1864,49 +1868,49 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>1238</t>
+          <t>1239</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>IH1238</t>
+          <t>IH1239</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>112L Bottom</t>
+          <t>110R</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>112L</t>
+          <t>110R</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>S</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1238</t>
+          <t>track/signalhead/IH1239</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; Digicon mast '112L'</t>
+          <t>LCOS Signal 7 UID 39; Digicon mast '110R'</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>C7-OU3-2</t>
+          <t>C7-OU3-3</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1926,49 +1930,49 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1239</t>
+          <t>1240</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>IH1239</t>
+          <t>IH1240</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>110R</t>
+          <t>112R Top</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>110R</t>
+          <t>112R</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>T</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1239</t>
+          <t>track/signalhead/IH1240</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; Digicon mast '110R'</t>
+          <t>LCOS Signal 8 UID 40; Digicon mast '112R'</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>C7-OU3-3</t>
+          <t>C7-OU3-4</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1988,22 +1992,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1240</t>
+          <t>1241</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>IH1240</t>
+          <t>IH1241</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>112R Top</t>
+          <t>112R Bottom</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2013,86 +2017,86 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1240</t>
+          <t>track/signalhead/IH1241</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>LCOS Signal 8 UID 40; Digicon mast '112R'</t>
+          <t>LCOS Signal 9 UID 41; Digicon mast '112R'</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>C7-OU3-4</t>
+          <t>D1-OU2-1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>North - Upper (East End)</t>
+          <t>Princess / Helix DCC node</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>1241</t>
+          <t>132</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>IH1241</t>
+          <t>IH132</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>112R Bottom</t>
+          <t>115LB Top</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>112R</t>
+          <t>115LB</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1241</t>
+          <t>track/signalhead/IH132</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>LCOS Signal 9 UID 41; Digicon mast '112R'</t>
+          <t>LCOS Signal 0 UID 32; Digicon mast '115LB'</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>D1-OU2-1</t>
+          <t>D1-OU2-2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2112,22 +2116,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>133</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>IH132</t>
+          <t>IH133</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>115LB Top</t>
+          <t>115LB Bottom</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2137,24 +2141,24 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>track/signalhead/IH132</t>
+          <t>track/signalhead/IH133</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; Digicon mast '115LB'</t>
+          <t>LCOS Signal 1 UID 33; Digicon mast '115LB'</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>D1-OU2-2</t>
+          <t>D1-OU2-3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2174,49 +2178,49 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>133</t>
+          <t>134</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>IH133</t>
+          <t>IH134</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>115LB Bottom</t>
+          <t>120R</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>115LB</t>
+          <t>120R</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>S</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>track/signalhead/IH133</t>
+          <t>track/signalhead/IH134</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; Digicon mast '115LB'</t>
+          <t>LCOS Signal 2 UID 34; Digicon mast '120R'</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>D1-OU2-3</t>
+          <t>D1-OU2-4</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2236,49 +2240,49 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>135</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>IH134</t>
+          <t>IH135</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>114R</t>
+          <t>113RA Top</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>114R</t>
+          <t>113RA</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>T</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>track/signalhead/IH134</t>
+          <t>track/signalhead/IH135</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; Digicon mast '114R'</t>
+          <t>LCOS Signal 3 UID 35; Digicon mast '113RA'</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>D1-OU2-4</t>
+          <t>D1-OU2-5</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2298,22 +2302,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>136</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>IH135</t>
+          <t>IH136</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>113RA Top</t>
+          <t>113RA Bottom</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2323,24 +2327,24 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>track/signalhead/IH135</t>
+          <t>track/signalhead/IH136</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; Digicon mast '113RA'</t>
+          <t>LCOS Signal 4 UID 36; Digicon mast '113RA'</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>D1-OU2-5</t>
+          <t>D1-OU2-6</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2360,49 +2364,49 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>137</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>IH136</t>
+          <t>IH137</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>113RA Bottom</t>
+          <t>113RB Top</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>113RA</t>
+          <t>113RB</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>track/signalhead/IH136</t>
+          <t>track/signalhead/IH137</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; Digicon mast '113RA'</t>
+          <t>LCOS Signal 5 UID 37; Digicon mast '113RB'</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>D1-OU2-6</t>
+          <t>D1-OU2-7</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2422,22 +2426,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>138</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>IH137</t>
+          <t>IH138</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>113RB Top</t>
+          <t>113RB Bottom</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2447,24 +2451,24 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>track/signalhead/IH137</t>
+          <t>track/signalhead/IH138</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; Digicon mast '113RB'</t>
+          <t>LCOS Signal 6 UID 38; Digicon mast '113RB'</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>D1-OU2-7</t>
+          <t>D1-OU2-8</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2484,49 +2488,49 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>139</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>IH138</t>
+          <t>IH139</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>113RB Bottom</t>
+          <t>114LB Top</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>113RB</t>
+          <t>114LB</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>track/signalhead/IH138</t>
+          <t>track/signalhead/IH139</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; Digicon mast '113RB'</t>
+          <t>LCOS Signal 7 UID 39; Digicon mast '114LB'</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>D1-OU2-8</t>
+          <t>D1-OU3-1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2546,22 +2550,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>140</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>IH139</t>
+          <t>IH140</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>114LB Top</t>
+          <t>114LB Bottom</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2571,24 +2575,24 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>track/signalhead/IH139</t>
+          <t>track/signalhead/IH140</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; Digicon mast '114LB'</t>
+          <t>LCOS Signal 8 UID 40; Digicon mast '114LB'</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>D1-OU3-1</t>
+          <t>D1-OU3-2</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2608,49 +2612,49 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>141</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>IH140</t>
+          <t>IH141</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>114LB Bottom</t>
+          <t>120L</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>114LB</t>
+          <t>120L</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>S</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>track/signalhead/IH140</t>
+          <t>track/signalhead/IH141</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>LCOS Signal 8 UID 40; Digicon mast '114LB'</t>
+          <t>LCOS Signal 9 UID 41; Digicon mast '120L'</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>D1-OU3-2</t>
+          <t>D1-OU3-3</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2670,27 +2674,27 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>142</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>IH141</t>
+          <t>IH142</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>115R</t>
+          <t>115LA</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>115R</t>
+          <t>115LA</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2700,19 +2704,19 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>track/signalhead/IH141</t>
+          <t>track/signalhead/IH142</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>LCOS Signal 9 UID 41; Digicon mast '115R'</t>
+          <t>LCOS Signal 10 UID 42; Digicon mast '115LA'</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>D1-OU3-3</t>
+          <t>D1-OU3-4</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2732,27 +2736,27 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>143</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>IH142</t>
+          <t>IH143</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>115LA</t>
+          <t>114LA</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>115LA</t>
+          <t>114LA</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2762,140 +2766,130 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>track/signalhead/IH142</t>
+          <t>track/signalhead/IH143</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>LCOS Signal 10 UID 42; Digicon mast '115LA'</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>D1-OU3-4</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Princess / Helix DCC node</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>143</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>IH143</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>114LA</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>114LA</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>track/signalhead/IH143</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
           <t>LCOS Signal 11 UID 43; Digicon mast '114LA'</t>
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Masts (cats/data/signal_head_plan.csv)</t>
+        </is>
+      </c>
+    </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>Masts (cats/data/signal_head_plan.csv)</t>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>mast_user_name</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>mqtt_node</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>parent_node_id</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>heads</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>appearance</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>physignal</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>mast_system_name</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>head_system_names</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>packed_ids</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>port_ids</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>mast_user_name</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>mqtt_node</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>parent_node_id</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>heads</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>appearance</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>physignal</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>mast_system_name</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>head_system_names</t>
-        </is>
-      </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t>packed_ids</t>
-        </is>
-      </c>
-      <c r="J43" s="3" t="inlineStr">
-        <is>
-          <t>port_ids</t>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>102LB</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SL-2-high-abs</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH432)(IH433)</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>IH432 IH433</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>432 433</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>C4-OU2-1 C4-OU2-2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>102LB</t>
+          <t>102LA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2910,44 +2904,44 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SL-2-high-abs</t>
+          <t>SL-1-low</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH432)(IH433)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH434)</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>IH432 IH433</t>
+          <t>IH434</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>432 433</t>
+          <t>434</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>C4-OU2-1 C4-OU2-2</t>
+          <t>C4-OU2-3</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>102LA</t>
+          <t>101RA</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2977,29 +2971,29 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH434)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH436)</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>IH434</t>
+          <t>IH436</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>434</t>
+          <t>436</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>C4-OU2-3</t>
+          <t>C4-OU2-5</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>101RA</t>
+          <t>101RB</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3029,29 +3023,29 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH436)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH437)</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>IH436</t>
+          <t>IH437</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>436</t>
+          <t>437</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>C4-OU2-5</t>
+          <t>C4-OU2-6</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>101RB</t>
+          <t>100L</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3066,54 +3060,54 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>SL-2-high-abs</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH437)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH438)(IH439)</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>IH437</t>
+          <t>IH438 IH439</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>437</t>
+          <t>438 439</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>C4-OU2-6</t>
+          <t>C4-OU3-1 C4-OU3-2</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>100L</t>
+          <t>117RA</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3133,29 +3127,29 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH438)(IH439)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1332)(IH1333)</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>IH438 IH439</t>
+          <t>IH1332 IH1333</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>438 439</t>
+          <t>1332 1333</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>C4-OU3-1 C4-OU3-2</t>
+          <t>C1-OU2-1 C1-OU2-2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>117RA</t>
+          <t>117LB</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3170,44 +3164,44 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SL-2-high-abs</t>
+          <t>SL-1-low</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1332)(IH1333)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH1334)</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>IH1332 IH1333</t>
+          <t>IH1334</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>1332 1333</t>
+          <t>1334</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>C1-OU2-1 C1-OU2-2</t>
+          <t>C1-OU2-3</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>117LB</t>
+          <t>117RB</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3222,44 +3216,44 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>SL-2-high-abs</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1334)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1335)(IH1336)</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>IH1334</t>
+          <t>IH1335 IH1336</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>1334</t>
+          <t>1335 1336</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>C1-OU2-3</t>
+          <t>C1-OU2-4 C1-OU2-5</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>117RB</t>
+          <t>117LA</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3289,39 +3283,39 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1335)(IH1336)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1337)(IH1338)</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>IH1335 IH1336</t>
+          <t>IH1337 IH1338</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>1335 1336</t>
+          <t>1337 1338</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>C1-OU2-4 C1-OU2-5</t>
+          <t>C1-OU2-6 C1-OU3-1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>117LA</t>
+          <t>111RA</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3341,29 +3335,29 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1337)(IH1338)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1232)(IH1233)</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>IH1337 IH1338</t>
+          <t>IH1232 IH1233</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>1337 1338</t>
+          <t>1232 1233</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>C1-OU2-6 C1-OU3-1</t>
+          <t>C7-OU2-1 C7-OU2-2</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>111RA</t>
+          <t>111L</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3393,29 +3387,29 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1232)(IH1233)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1234)(IH1235)</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>IH1232 IH1233</t>
+          <t>IH1234 IH1235</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>1232 1233</t>
+          <t>1234 1235</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>C7-OU2-1 C7-OU2-2</t>
+          <t>C7-OU2-3 C7-OU2-4</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>111L</t>
+          <t>111RB</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3430,44 +3424,44 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SL-2-high-abs</t>
+          <t>SL-1-low</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1234)(IH1235)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH1236)</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>IH1234 IH1235</t>
+          <t>IH1236</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>1234 1235</t>
+          <t>1236</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>C7-OU2-3 C7-OU2-4</t>
+          <t>C7-OU2-5</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>111RB</t>
+          <t>112L</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3482,44 +3476,44 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>SL-2-high-abs</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1236)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1237)(IH1238)</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>IH1236</t>
+          <t>IH1237 IH1238</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>1236</t>
+          <t>1237 1238</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>C7-OU2-5</t>
+          <t>C7-OU2-6 C7-OU3-1</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>112L</t>
+          <t>110R</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3534,44 +3528,44 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>SL-2-high-abs</t>
+          <t>SL-1-low</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1237)(IH1238)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH1239)</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>IH1237 IH1238</t>
+          <t>IH1239</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>1237 1238</t>
+          <t>1239</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>C7-OU2-6 C7-OU3-1</t>
+          <t>C7-OU3-2</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>110R</t>
+          <t>112R</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3586,54 +3580,54 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>SL-2-high-abs</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1239)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1240)(IH1241)</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>IH1239</t>
+          <t>IH1240 IH1241</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>1239</t>
+          <t>1240 1241</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>C7-OU3-2</t>
+          <t>C7-OU3-3 C7-OU3-4</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>112R</t>
+          <t>115LB</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3653,29 +3647,29 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1240)(IH1241)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH132)(IH133)</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>IH1240 IH1241</t>
+          <t>IH132 IH133</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>1240 1241</t>
+          <t>132 133</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>C7-OU3-3 C7-OU3-4</t>
+          <t>D1-OU2-1 D1-OU2-2</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>115LB</t>
+          <t>120R</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3690,44 +3684,44 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>SL-2-high-abs</t>
+          <t>SL-1-low</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH132)(IH133)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH134)</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>IH132 IH133</t>
+          <t>IH134</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>132 133</t>
+          <t>134</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>D1-OU2-1 D1-OU2-2</t>
+          <t>D1-OU2-3</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>114R</t>
+          <t>113RA</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3742,44 +3736,44 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>SL-2-high-abs</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH134)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH135)(IH136)</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>IH134</t>
+          <t>IH135 IH136</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>135 136</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>D1-OU2-3</t>
+          <t>D1-OU2-4 D1-OU2-5</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>113RA</t>
+          <t>113RB</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3809,29 +3803,29 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH135)(IH136)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH137)(IH138)</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>IH135 IH136</t>
+          <t>IH137 IH138</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>135 136</t>
+          <t>137 138</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>D1-OU2-4 D1-OU2-5</t>
+          <t>D1-OU2-6 D1-OU2-7</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>113RB</t>
+          <t>114LB</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3861,29 +3855,29 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH137)(IH138)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH139)(IH140)</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>IH137 IH138</t>
+          <t>IH139 IH140</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>137 138</t>
+          <t>139 140</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>D1-OU2-6 D1-OU2-7</t>
+          <t>D1-OU2-8 D1-OU3-1</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>114LB</t>
+          <t>120L</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3898,44 +3892,44 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>SL-2-high-abs</t>
+          <t>SL-1-low</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH139)(IH140)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH141)</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>IH139 IH140</t>
+          <t>IH141</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>139 140</t>
+          <t>141</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>D1-OU2-8 D1-OU3-1</t>
+          <t>D1-OU3-2</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>115R</t>
+          <t>115LA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3965,29 +3959,29 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH141)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH142)</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>IH141</t>
+          <t>IH142</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>142</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>D1-OU3-2</t>
+          <t>D1-OU3-3</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>115LA</t>
+          <t>114LA</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -4017,72 +4011,20 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH142)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH143)</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>IH142</t>
+          <t>IH143</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>143</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
-        <is>
-          <t>D1-OU3-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>114LA</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>SL-1-low</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>single</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH143)</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>IH143</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>143</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
         <is>
           <t>D1-OU3-4</t>
         </is>
@@ -8988,22 +8930,17 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>spare C4-OU2-4</t>
+          <t>S3-7 G</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Signal LED</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
           <t>5V</t>
-        </is>
-      </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>HART Digicon searchlight; MQTT track/signalhead/IH435; packed 435 (node 4 sig 3); was S3-7 G</t>
         </is>
       </c>
     </row>
@@ -17138,7 +17075,7 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>114R</t>
+          <t>120R</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
@@ -17418,7 +17355,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>115R</t>
+          <t>120L</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
@@ -23038,7 +22975,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>114R</t>
+          <t>120R</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -23125,7 +23062,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>115R</t>
+          <t>120L</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">

</xml_diff>

<commit_message>
Apply CTC public names (Switch 1, Mast 2L, OS S-R, Mast 2035/2036) and refresh wiring docs.
Keep MQTT systemNames and ISNX frozen; rewire CATS Master 4 and USS v74; restamp Desktop v85. Re-Discover SML after reload.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
+++ b/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
@@ -581,12 +581,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>102LB Top</t>
+          <t>Head 6LB Top</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>102LB</t>
+          <t>Mast 6LB</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; Digicon mast '102LB'</t>
+          <t>LCOS Signal 0 UID 32; Digicon mast '6LB'</t>
         </is>
       </c>
     </row>
@@ -643,12 +643,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>102LB Bottom</t>
+          <t>Head 6LB Bottom</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>102LB</t>
+          <t>Mast 6LB</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; Digicon mast '102LB'</t>
+          <t>LCOS Signal 1 UID 33; Digicon mast '6LB'</t>
         </is>
       </c>
     </row>
@@ -705,12 +705,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>102LA</t>
+          <t>Head 6LA</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>102LA</t>
+          <t>Mast 6LA</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; Digicon mast '102LA' (1-head; was Top of 2-head)</t>
+          <t>LCOS Signal 2 UID 34; Digicon mast '6LA' (1-head; was Top of 2-head)</t>
         </is>
       </c>
     </row>
@@ -767,12 +767,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>101RA</t>
+          <t>Head 4RA</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>101RA</t>
+          <t>Mast 4RA</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; Digicon mast '101RA'</t>
+          <t>LCOS Signal 4 UID 36; Digicon mast '4RA'</t>
         </is>
       </c>
     </row>
@@ -829,12 +829,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>101RB</t>
+          <t>Head 4RB</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>101RB</t>
+          <t>Mast 4RB</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; Digicon mast '101RB'</t>
+          <t>LCOS Signal 5 UID 37; Digicon mast '4RB'</t>
         </is>
       </c>
     </row>
@@ -891,12 +891,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>100L Top</t>
+          <t>Head 2L Top</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>100L</t>
+          <t>Mast 2L</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; Digicon mast '100L'</t>
+          <t>LCOS Signal 6 UID 38; Digicon mast '2L'</t>
         </is>
       </c>
     </row>
@@ -953,12 +953,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>100L Bottom</t>
+          <t>Head 2L Bottom</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>100L</t>
+          <t>Mast 2L</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; Digicon mast '100L'</t>
+          <t>LCOS Signal 7 UID 39; Digicon mast '2L'</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1015,12 +1015,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>117RA Top</t>
+          <t>Head 8RA Top</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>117RA</t>
+          <t>Mast 8RA</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; Digicon mast '117RA'</t>
+          <t>LCOS Signal 0 UID 32; Digicon mast '8RA'</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1077,12 +1077,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>117RA Bottom</t>
+          <t>Head 8RA Bottom</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>117RA</t>
+          <t>Mast 8RA</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; Digicon mast '117RA'</t>
+          <t>LCOS Signal 1 UID 33; Digicon mast '8RA'</t>
         </is>
       </c>
     </row>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1139,12 +1139,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>117LB</t>
+          <t>Head 8LB</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>117LB</t>
+          <t>Mast 8LB</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; Digicon mast '117LB'</t>
+          <t>LCOS Signal 2 UID 34; Digicon mast '8LB'</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1201,12 +1201,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>117RB Top</t>
+          <t>Head 8RB Top</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>117RB</t>
+          <t>Mast 8RB</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; Digicon mast '117RB'</t>
+          <t>LCOS Signal 3 UID 35; Digicon mast '8RB'</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1263,12 +1263,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>117RB Bottom</t>
+          <t>Head 8RB Bottom</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>117RB</t>
+          <t>Mast 8RB</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; Digicon mast '117RB'</t>
+          <t>LCOS Signal 4 UID 36; Digicon mast '8RB'</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1325,12 +1325,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>117LA Top</t>
+          <t>Head 8LA Top</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>117LA</t>
+          <t>Mast 8LA</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; Digicon mast '117LA'</t>
+          <t>LCOS Signal 5 UID 37; Digicon mast '8LA'</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1387,12 +1387,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>117LA Bottom</t>
+          <t>Head 8LA Bottom</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>117LA</t>
+          <t>Mast 8LA</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; Digicon mast '117LA'</t>
+          <t>LCOS Signal 6 UID 38; Digicon mast '8LA'</t>
         </is>
       </c>
     </row>
@@ -1449,12 +1449,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>111RA Top</t>
+          <t>Head 24RA Top</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>111RA</t>
+          <t>Mast 24RA</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; Digicon mast '111RA'</t>
+          <t>LCOS Signal 0 UID 32; Digicon mast '24RA'</t>
         </is>
       </c>
     </row>
@@ -1511,12 +1511,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>111RA Bottom</t>
+          <t>Head 24RA Bottom</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>111RA</t>
+          <t>Mast 24RA</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; Digicon mast '111RA'</t>
+          <t>LCOS Signal 1 UID 33; Digicon mast '24RA'</t>
         </is>
       </c>
     </row>
@@ -1573,12 +1573,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>111L Top</t>
+          <t>Head 24L Top</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>111L</t>
+          <t>Mast 24L</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; Digicon mast '111L'</t>
+          <t>LCOS Signal 2 UID 34; Digicon mast '24L'</t>
         </is>
       </c>
     </row>
@@ -1635,12 +1635,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>111L Bottom</t>
+          <t>Head 24L Bottom</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>111L</t>
+          <t>Mast 24L</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; Digicon mast '111L'</t>
+          <t>LCOS Signal 3 UID 35; Digicon mast '24L'</t>
         </is>
       </c>
     </row>
@@ -1697,12 +1697,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>111RB</t>
+          <t>Head 24RB</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>111RB</t>
+          <t>Mast 24RB</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; Digicon mast '111RB'</t>
+          <t>LCOS Signal 4 UID 36; Digicon mast '24RB'</t>
         </is>
       </c>
     </row>
@@ -1759,12 +1759,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>112L Top</t>
+          <t>Head 34L Top</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>112L</t>
+          <t>Mast 34L</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; Digicon mast '112L'</t>
+          <t>LCOS Signal 5 UID 37; Digicon mast '34L'</t>
         </is>
       </c>
     </row>
@@ -1821,12 +1821,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>112L Bottom</t>
+          <t>Head 34L Bottom</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>112L</t>
+          <t>Mast 34L</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; Digicon mast '112L'</t>
+          <t>LCOS Signal 6 UID 38; Digicon mast '34L'</t>
         </is>
       </c>
     </row>
@@ -1883,12 +1883,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>110R</t>
+          <t>Head 32R</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>110R</t>
+          <t>Mast 32R</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; Digicon mast '110R'</t>
+          <t>LCOS Signal 7 UID 39; Digicon mast '32R'</t>
         </is>
       </c>
     </row>
@@ -1945,12 +1945,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>112R Top</t>
+          <t>Head 34R Top</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>112R</t>
+          <t>Mast 34R</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>LCOS Signal 8 UID 40; Digicon mast '112R'</t>
+          <t>LCOS Signal 8 UID 40; Digicon mast '34R'</t>
         </is>
       </c>
     </row>
@@ -2007,12 +2007,12 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>112R Bottom</t>
+          <t>Head 34R Bottom</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>112R</t>
+          <t>Mast 34R</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>LCOS Signal 9 UID 41; Digicon mast '112R'</t>
+          <t>LCOS Signal 9 UID 41; Digicon mast '34R'</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>115LB Top</t>
+          <t>Head 40LB Top</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>115LB</t>
+          <t>Mast 40LB</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; Digicon mast '115LB'</t>
+          <t>LCOS Signal 0 UID 32; Digicon mast '40LB'</t>
         </is>
       </c>
     </row>
@@ -2131,12 +2131,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>115LB Bottom</t>
+          <t>Head 40LB Bottom</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>115LB</t>
+          <t>Mast 40LB</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; Digicon mast '115LB'</t>
+          <t>LCOS Signal 1 UID 33; Digicon mast '40LB'</t>
         </is>
       </c>
     </row>
@@ -2193,12 +2193,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>120R</t>
+          <t>Head 2036</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>120R</t>
+          <t>Mast 2036</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; Digicon mast '120R'</t>
+          <t>LCOS Signal 2 UID 34; Digicon mast '2036'</t>
         </is>
       </c>
     </row>
@@ -2255,12 +2255,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>113RA Top</t>
+          <t>Head 36RA Top</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>113RA</t>
+          <t>Mast 36RA</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; Digicon mast '113RA'</t>
+          <t>LCOS Signal 3 UID 35; Digicon mast '36RA'</t>
         </is>
       </c>
     </row>
@@ -2317,12 +2317,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>113RA Bottom</t>
+          <t>Head 36RA Bottom</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>113RA</t>
+          <t>Mast 36RA</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; Digicon mast '113RA'</t>
+          <t>LCOS Signal 4 UID 36; Digicon mast '36RA'</t>
         </is>
       </c>
     </row>
@@ -2379,12 +2379,12 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>113RB Top</t>
+          <t>Head 36RB Top</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>113RB</t>
+          <t>Mast 36RB</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; Digicon mast '113RB'</t>
+          <t>LCOS Signal 5 UID 37; Digicon mast '36RB'</t>
         </is>
       </c>
     </row>
@@ -2441,12 +2441,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>113RB Bottom</t>
+          <t>Head 36RB Bottom</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>113RB</t>
+          <t>Mast 36RB</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2461,7 +2461,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; Digicon mast '113RB'</t>
+          <t>LCOS Signal 6 UID 38; Digicon mast '36RB'</t>
         </is>
       </c>
     </row>
@@ -2503,12 +2503,12 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>114LB Top</t>
+          <t>Head 38LB Top</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>114LB</t>
+          <t>Mast 38LB</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2523,7 +2523,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; Digicon mast '114LB'</t>
+          <t>LCOS Signal 7 UID 39; Digicon mast '38LB'</t>
         </is>
       </c>
     </row>
@@ -2565,12 +2565,12 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>114LB Bottom</t>
+          <t>Head 38LB Bottom</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>114LB</t>
+          <t>Mast 38LB</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>LCOS Signal 8 UID 40; Digicon mast '114LB'</t>
+          <t>LCOS Signal 8 UID 40; Digicon mast '38LB'</t>
         </is>
       </c>
     </row>
@@ -2627,12 +2627,12 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>120L</t>
+          <t>Head 2035</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>120L</t>
+          <t>Mast 2035</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>LCOS Signal 9 UID 41; Digicon mast '120L'</t>
+          <t>LCOS Signal 9 UID 41; Digicon mast '2035'</t>
         </is>
       </c>
     </row>
@@ -2689,12 +2689,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>115LA</t>
+          <t>Head 40LA</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>115LA</t>
+          <t>Mast 40LA</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>LCOS Signal 10 UID 42; Digicon mast '115LA'</t>
+          <t>LCOS Signal 10 UID 42; Digicon mast '40LA'</t>
         </is>
       </c>
     </row>
@@ -2751,12 +2751,12 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>114LA</t>
+          <t>Head 38LA</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>114LA</t>
+          <t>Mast 38LA</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>LCOS Signal 11 UID 43; Digicon mast '114LA'</t>
+          <t>LCOS Signal 11 UID 43; Digicon mast '38LA'</t>
         </is>
       </c>
     </row>
@@ -2837,7 +2837,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>102LB</t>
+          <t>Mast 6LB</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2889,7 +2889,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>102LA</t>
+          <t>Mast 6LA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2941,7 +2941,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>101RA</t>
+          <t>Mast 4RA</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2993,7 +2993,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>101RB</t>
+          <t>Mast 4RB</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3045,7 +3045,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>100L</t>
+          <t>Mast 2L</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3097,7 +3097,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>117RA</t>
+          <t>Mast 8RA</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3149,7 +3149,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>117LB</t>
+          <t>Mast 8LB</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3201,7 +3201,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>117RB</t>
+          <t>Mast 8RB</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3253,7 +3253,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>117LA</t>
+          <t>Mast 8LA</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3305,7 +3305,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>111RA</t>
+          <t>Mast 24RA</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3357,7 +3357,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>111L</t>
+          <t>Mast 24L</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3409,7 +3409,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>111RB</t>
+          <t>Mast 24RB</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3461,7 +3461,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>112L</t>
+          <t>Mast 34L</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3513,7 +3513,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>110R</t>
+          <t>Mast 32R</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3565,7 +3565,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>112R</t>
+          <t>Mast 34R</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>115LB</t>
+          <t>Mast 40LB</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3669,7 +3669,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>120R</t>
+          <t>Mast 2036</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3721,7 +3721,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>113RA</t>
+          <t>Mast 36RA</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3773,7 +3773,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>113RB</t>
+          <t>Mast 36RB</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3825,7 +3825,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>114LB</t>
+          <t>Mast 38LB</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3877,7 +3877,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>120L</t>
+          <t>Mast 2035</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3929,7 +3929,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>115LA</t>
+          <t>Mast 40LA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3981,7 +3981,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>114LA</t>
+          <t>Mast 38LA</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -6267,7 +6267,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -6275,7 +6275,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>117RA Top</t>
+          <t>Head 8RA Top</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -6307,7 +6307,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -6315,7 +6315,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>117RA Bottom</t>
+          <t>Head 8RA Bottom</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -6347,7 +6347,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -6355,7 +6355,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>117LB</t>
+          <t>Head 8LB</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -6387,7 +6387,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>117RB Top</t>
+          <t>Head 8RB Top</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>117RB Bottom</t>
+          <t>Head 8RB Bottom</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -6467,7 +6467,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -6475,7 +6475,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>117LA Top</t>
+          <t>Head 8LA Top</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -6567,7 +6567,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Helix - Lower (Barn / West Yard)</t>
+          <t>Helix - Lower (OS Barn / West Yard)</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -6575,7 +6575,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>117LA Bottom</t>
+          <t>Head 8LA Bottom</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -8810,7 +8810,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>102LB Top</t>
+          <t>Head 6LB Top</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -8850,7 +8850,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>102LB Bottom</t>
+          <t>Head 6LB Bottom</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -8890,7 +8890,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>102LA</t>
+          <t>Head 6LA</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -8965,7 +8965,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>101RA</t>
+          <t>Head 4RA</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -9005,7 +9005,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>101RB</t>
+          <t>Head 4RB</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -9115,7 +9115,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>100L Top</t>
+          <t>Head 2L Top</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -9155,7 +9155,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>100L Bottom</t>
+          <t>Head 2L Bottom</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -11095,7 +11095,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>111RA Top</t>
+          <t>Head 24RA Top</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -11135,7 +11135,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>111RA Bottom</t>
+          <t>Head 24RA Bottom</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -11175,7 +11175,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>111L Top</t>
+          <t>Head 24L Top</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -11215,7 +11215,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>111L Bottom</t>
+          <t>Head 24L Bottom</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -11255,7 +11255,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>111RB</t>
+          <t>Head 24RB</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>112L Top</t>
+          <t>Head 34L Top</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -11395,7 +11395,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>112L Bottom</t>
+          <t>Head 34L Bottom</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -11435,7 +11435,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>110R</t>
+          <t>Head 32R</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -11475,7 +11475,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>112R Top</t>
+          <t>Head 34R Top</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -11515,7 +11515,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>112R Bottom</t>
+          <t>Head 34R Bottom</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -16995,7 +16995,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>115LB Top</t>
+          <t>Head 40LB Top</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -17035,7 +17035,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>115LB Bottom</t>
+          <t>Head 40LB Bottom</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
@@ -17075,7 +17075,7 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>120R</t>
+          <t>Head 2036</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
@@ -17115,7 +17115,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>113RA Top</t>
+          <t>Head 36RA Top</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
@@ -17155,7 +17155,7 @@
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>113RA Bottom</t>
+          <t>Head 36RA Bottom</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
@@ -17195,7 +17195,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>113RB Top</t>
+          <t>Head 36RB Top</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
@@ -17235,7 +17235,7 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>113RB Bottom</t>
+          <t>Head 36RB Bottom</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
@@ -17275,7 +17275,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>114LB Top</t>
+          <t>Head 38LB Top</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
@@ -17315,7 +17315,7 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>114LB Bottom</t>
+          <t>Head 38LB Bottom</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
@@ -17355,7 +17355,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>120L</t>
+          <t>Head 2035</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
@@ -17395,7 +17395,7 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>115LA</t>
+          <t>Head 40LA</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
@@ -17435,7 +17435,7 @@
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>114LA</t>
+          <t>Head 38LA</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
@@ -22848,7 +22848,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Switch 113</t>
+          <t>Switch 35</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -22883,7 +22883,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>113RA</t>
+          <t>Mast 36RA</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -22918,7 +22918,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>113RB</t>
+          <t>Mast 36RB</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -22940,24 +22940,24 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Switch 37</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Helix - Lower</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Switch 114</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Helix - Lower</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Switch 114</t>
-        </is>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>C1-IN2-2</t>
@@ -22975,7 +22975,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>120R</t>
+          <t>Head 2036</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -22985,7 +22985,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>114LB</t>
+          <t>Mast 38LB</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -23005,7 +23005,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>114LA</t>
+          <t>Head 38LA</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -23027,24 +23027,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Switch 39</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Helix - Lower</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>Switch 115</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Helix - Lower</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Switch 115</t>
-        </is>
-      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>C1-IN2-3</t>
@@ -23062,7 +23062,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>120L</t>
+          <t>Head 2035</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -23072,12 +23072,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>115LB</t>
+          <t>Mast 40LB</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>115LA</t>
+          <t>Head 40LA</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -23196,7 +23196,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Switch 111</t>
+          <t>Switch 23</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -23231,7 +23231,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>111L</t>
+          <t>Mast 24L</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -23246,7 +23246,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>111RA</t>
+          <t>Mast 24RA</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -23266,7 +23266,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>111RB</t>
+          <t>Head 24RB</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -23288,24 +23288,24 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Switch 33</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>North - Lower</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>Switch 112</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>North - Lower</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Switch 112</t>
-        </is>
-      </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>C2-IN2-6</t>
@@ -23323,7 +23323,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>112L</t>
+          <t>Mast 34L</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -23338,7 +23338,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>112R</t>
+          <t>Mast 34R</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -23437,24 +23437,24 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Switch 31</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>North - Lower</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>Switch 110</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>North - Lower</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Switch 110</t>
-        </is>
-      </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>C2-IN2-4</t>
@@ -23472,7 +23472,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>110R</t>
+          <t>Head 32R</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -23889,24 +23889,24 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>Switch 1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Peninsula - Lower</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>Switch 100</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>C6</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Peninsula - Lower</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Switch 100</t>
-        </is>
-      </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>C6-IN2-1</t>
@@ -23924,7 +23924,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>100L</t>
+          <t>Mast 2L</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -23941,24 +23941,24 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Switch 3</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Peninsula - Lower</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>Switch 101</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>C6</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Peninsula - Lower</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Switch 101</t>
-        </is>
-      </c>
       <c r="E19" t="inlineStr">
         <is>
           <t>C6-IN2-2</t>
@@ -23996,7 +23996,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>101RA</t>
+          <t>Head 4RA</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -24016,31 +24016,31 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>101RB</t>
+          <t>Head 4RB</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Switch 5</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Peninsula - Lower</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>Switch 102</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>C6</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Peninsula - Lower</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Switch 102</t>
-        </is>
-      </c>
       <c r="E20" t="inlineStr">
         <is>
           <t>C6-IN2-3</t>
@@ -24058,7 +24058,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>102LA</t>
+          <t>Head 6LA</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -24088,7 +24088,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>102LB</t>
+          <t>Mast 6LB</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -24988,7 +24988,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Switch 117</t>
+          <t>Switch 7</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -25023,7 +25023,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>117RA</t>
+          <t>Mast 8RA</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -25038,12 +25038,12 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>117LA</t>
+          <t>Mast 8LA</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>117LB / 117RB</t>
+          <t>Head 8LB / Mast 8RB</t>
         </is>
       </c>
     </row>
@@ -25204,7 +25204,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OS 101</t>
+          <t>OS 3</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -25249,7 +25249,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OS 100</t>
+          <t>OS 1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -25294,7 +25294,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>W-2</t>
+          <t>OS W-2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -25339,7 +25339,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>W-1</t>
+          <t>OS W-1</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -25384,7 +25384,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>OS 102</t>
+          <t>OS 5</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -25429,7 +25429,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Brick-Plane</t>
+          <t>OS Brick-Plane</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -25474,7 +25474,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>East Main Ext</t>
+          <t>OS East Main Ext</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -25519,7 +25519,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Scale</t>
+          <t>OS Scale</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -25564,7 +25564,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>OS 116</t>
+          <t>OS 13</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -25609,7 +25609,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OS 103</t>
+          <t>OS 15</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -25654,7 +25654,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OS 104</t>
+          <t>OS 17</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -25744,7 +25744,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OS 105</t>
+          <t>OS 19</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -25834,7 +25834,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>OS 106</t>
+          <t>OS 21</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -25924,7 +25924,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Main West</t>
+          <t>OS Main West</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -26014,7 +26014,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Main East</t>
+          <t>OS Main East</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -26059,7 +26059,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>S-5</t>
+          <t>OS S-4</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -26104,7 +26104,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>S-4</t>
+          <t>OS S-3</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -26149,7 +26149,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>S-3</t>
+          <t>OS S-2</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -26194,7 +26194,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>S-2</t>
+          <t>OS S-1</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -26239,7 +26239,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>S-1</t>
+          <t>OS S-R</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -26284,7 +26284,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>OS 107</t>
+          <t>OS 25</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -26374,7 +26374,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>OS 108</t>
+          <t>OS 27</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -26419,7 +26419,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>OS 111a</t>
+          <t>OS 23a</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -26464,7 +26464,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>OS 109</t>
+          <t>OS 29</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -26509,7 +26509,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>OS 111b</t>
+          <t>OS 23b</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -26554,7 +26554,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>OS 110</t>
+          <t>OS 31</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -26599,7 +26599,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OS 112</t>
+          <t>OS 33</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -26644,7 +26644,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>McKees Rocks</t>
+          <t>OS McKees Rocks</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -26689,7 +26689,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>McKeesport</t>
+          <t>OS McKeesport</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -26734,7 +26734,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OS 114 / K-2</t>
+          <t>OS 37</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -26779,7 +26779,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>OS 115 / K-1</t>
+          <t>OS 39</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -26824,7 +26824,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>OS 113b</t>
+          <t>OS 35b</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -26869,7 +26869,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>OS 113a</t>
+          <t>OS 35a</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -26914,7 +26914,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>East Lead</t>
+          <t>OS East Lead</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -26959,7 +26959,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>West Main Ext</t>
+          <t>OS West Main Ext</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -28654,7 +28654,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Barn</t>
+          <t>OS Barn</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -28699,7 +28699,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>OS 118</t>
+          <t>OS 11</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -28744,7 +28744,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>OS 117</t>
+          <t>OS 7</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -28789,7 +28789,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>OS 117b</t>
+          <t>OS 7b</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -28834,7 +28834,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>EH-3</t>
+          <t>OS EH-3</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -28879,7 +28879,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>EH-2</t>
+          <t>OS EH-2</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -28924,7 +28924,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>EH-1</t>
+          <t>OS EH-1</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -28969,7 +28969,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>OS 119</t>
+          <t>OS 9</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">

</xml_diff>

<commit_message>
Reserve pin 8 of the first 5V OU on every block-sensor node for detector calibration.
Digicon lamps that sat on those pins moved to the next leftover channel; relays that were there need a new home.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
+++ b/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
@@ -1053,14 +1053,14 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G/Y on Plane OU2; R spills to 2L OU3</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G on Plane OU2; Y/R on 2L OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C4-OU2-8</t>
+          <t>C4-OU3-8</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was G/Y on Plane OU2; R spills to 2L OU3</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was G on Plane OU2; Y/R on 2L OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was G/Y on Plane OU2; R spills to 2L OU3</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was G on Plane OU2; Y/R on 2L OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -4077,14 +4077,14 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G/Y with 24RA; R spills to 24L OU2</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G with 24RA; Y on OU3 (OU1-8 is BS cal); R with 24L</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>C2-OU1-8</t>
+          <t>C2-OU3-8</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -4149,7 +4149,7 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was G/Y with 24RA; R spills to 24L OU2</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was G with 24RA; Y on OU3 (OU1-8 is BS cal); R with 24L</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was G/Y with 24RA; R spills to 24L OU2</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was G with 24RA; Y on OU3 (OU1-8 is BS cal); R with 24L</t>
         </is>
       </c>
     </row>
@@ -5157,14 +5157,14 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G/Y with 34L; R spills to 34R OU3</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G with 34L; Y/R on 34R OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>C12-OU2-8</t>
+          <t>C12-OU3-8</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -5229,7 +5229,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was G/Y with 34L; R spills to 34R OU3</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was G with 34L; Y/R on 34R OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was G/Y with 34L; R spills to 34R OU3</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was G with 34L; Y/R on 34R OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -7749,14 +7749,14 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was G/Y with 40LB; R spills to balloon OU3</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was G with 40LB; Y/R on balloon OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>C11-OU2-8</t>
+          <t>C11-OU3-8</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -7821,7 +7821,7 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp Y; was G/Y with 40LB; R spills to balloon OU3</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp Y; was G with 40LB; Y/R on balloon OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -7893,7 +7893,7 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was G/Y with 40LB; R spills to balloon OU3</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was G with 40LB; Y/R on balloon OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -8488,7 +8488,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>C4-OU2-7 C4-OU2-8 C4-OU3-7</t>
+          <t>C4-OU2-7 C4-OU3-8 C4-OU3-7</t>
         </is>
       </c>
     </row>
@@ -8956,7 +8956,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>C2-OU1-7 C2-OU1-8 C2-OU2-7</t>
+          <t>C2-OU1-7 C2-OU3-8 C2-OU2-7</t>
         </is>
       </c>
     </row>
@@ -9112,7 +9112,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>C12-OU2-7 C12-OU2-8 C12-OU3-7</t>
+          <t>C12-OU2-7 C12-OU3-8 C12-OU3-7</t>
         </is>
       </c>
     </row>
@@ -9476,7 +9476,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>C11-OU2-7 C11-OU2-8 C11-OU3-7</t>
+          <t>C11-OU2-7 C11-OU3-8 C11-OU3-7</t>
         </is>
       </c>
     </row>
@@ -12189,17 +12189,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>C1 RELAY 1</t>
+          <t>Block sensor calibration</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Relay</t>
+          <t>Block Sensor Cal</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Block sensor calibration current (first 5V OU pin 8); not a lamp; was C1 RELAY 1</t>
         </is>
       </c>
     </row>
@@ -13106,7 +13111,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>North - Lower (East End 34)</t>
+          <t>North - Lower</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -13114,12 +13119,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Head 32R Y</t>
+          <t>Block sensor calibration</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Block Sensor Cal</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -13129,7 +13134,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1234; packed 1234 (node 12 sig 2); was C12 RELAY 1</t>
+          <t>Block sensor calibration current (first 5V OU pin 8); not a lamp; was C12 RELAY 1</t>
         </is>
       </c>
     </row>
@@ -13426,7 +13431,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>North - Lower</t>
+          <t>North - Lower (East End 34)</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -13434,17 +13439,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>S2-8 R</t>
+          <t>Head 32R Y</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Signal LED</t>
+          <t>Searchlight Signal Head</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1234; packed 1234 (node 12 sig 2); was S2-8 R</t>
         </is>
       </c>
     </row>
@@ -13741,7 +13751,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>North - Lower (East End west 24)</t>
+          <t>North - Lower</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -13749,12 +13759,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Head 24RB Y</t>
+          <t>Block sensor calibration</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Block Sensor Cal</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -13764,7 +13774,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
+          <t>Block sensor calibration current (first 5V OU pin 8); not a lamp</t>
         </is>
       </c>
     </row>
@@ -14321,15 +14331,30 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>North - Lower</t>
+          <t>North - Lower (East End west 24)</t>
         </is>
       </c>
       <c r="D73" t="n">
         <v>8</v>
       </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Head 24RB Y</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Searchlight Signal Head</t>
+        </is>
+      </c>
       <c r="G73" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
         </is>
       </c>
     </row>
@@ -14919,17 +14944,22 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>C3 RELAY 1</t>
+          <t>Block sensor calibration</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Relay</t>
+          <t>Block Sensor Cal</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Block sensor calibration current (first 5V OU pin 8); not a lamp; was C3 RELAY 1</t>
         </is>
       </c>
     </row>
@@ -15509,17 +15539,22 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>S3-14 R</t>
+          <t>Block sensor calibration</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Signal LED</t>
+          <t>Block Sensor Cal</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Block sensor calibration current (first 5V OU pin 8); not a lamp; was S3-14 R</t>
         </is>
       </c>
     </row>
@@ -16456,7 +16491,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>West - Lower (Plane)</t>
+          <t>Peninsula - Lower</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -16464,12 +16499,12 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Head 6LA Y</t>
+          <t>Block sensor calibration</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Block Sensor Cal</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -16479,7 +16514,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/434; packed 434 (node 4 sig 2); was C4 RELAY 1</t>
+          <t>Block sensor calibration current (first 5V OU pin 8); not a lamp; was C4 RELAY 1</t>
         </is>
       </c>
     </row>
@@ -16776,15 +16811,30 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Peninsula - Lower</t>
+          <t>West - Lower (Plane)</t>
         </is>
       </c>
       <c r="D137" t="n">
         <v>8</v>
       </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Head 6LA Y</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Searchlight Signal Head</t>
+        </is>
+      </c>
       <c r="G137" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/434; packed 434 (node 4 sig 2)</t>
         </is>
       </c>
     </row>
@@ -17371,7 +17421,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Helix (Princess east SW39)</t>
+          <t>Helix</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -17379,12 +17429,12 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Head 40LA Y</t>
+          <t>Block sensor calibration</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Block Sensor Cal</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -17394,7 +17444,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4); was C23 RELAY 1</t>
+          <t>Block sensor calibration current (first 5V OU pin 8); not a lamp; was C23 RELAY 1</t>
         </is>
       </c>
     </row>
@@ -17691,15 +17741,30 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Helix</t>
+          <t>Helix (Princess east SW39)</t>
         </is>
       </c>
       <c r="D161" t="n">
         <v>8</v>
       </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Head 40LA Y</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Searchlight Signal Head</t>
+        </is>
+      </c>
       <c r="G161" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4)</t>
         </is>
       </c>
     </row>
@@ -18249,17 +18314,22 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>C4 RELAY 1</t>
+          <t>Block sensor calibration</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Relay</t>
+          <t>Block Sensor Cal</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Block sensor calibration current (first 5V OU pin 8); not a lamp; was C4 RELAY 1</t>
         </is>
       </c>
     </row>
@@ -19089,17 +19159,22 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>C11 RELAY 1</t>
+          <t>Block sensor calibration</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Relay</t>
+          <t>Block Sensor Cal</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Block sensor calibration current (first 5V OU pin 8); not a lamp; was C11 RELAY 1</t>
         </is>
       </c>
     </row>
@@ -20419,17 +20494,22 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>C32 RELAY 1</t>
+          <t>Block sensor calibration</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>Relay</t>
+          <t>Block Sensor Cal</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>Block sensor calibration current (first 5V OU pin 8); not a lamp; was C32 RELAY 1</t>
         </is>
       </c>
     </row>
@@ -21299,17 +21379,22 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>C23 RELAY 1</t>
+          <t>Block sensor calibration</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>Relay</t>
+          <t>Block Sensor Cal</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>Block sensor calibration current (first 5V OU pin 8); not a lamp; was C23 RELAY 1</t>
         </is>
       </c>
     </row>
@@ -22169,17 +22254,22 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>C14 RELAY 1</t>
+          <t>Block sensor calibration</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>Relay</t>
+          <t>Block Sensor Cal</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Block sensor calibration current (first 5V OU pin 8); not a lamp; was C14 RELAY 1</t>
         </is>
       </c>
     </row>
@@ -30016,7 +30106,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>C12-OU2-8</t>
+          <t>C12-OU3-8</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -30617,7 +30707,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>C4-OU2-8</t>
+          <t>C4-OU3-8</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">

</xml_diff>

<commit_message>
Restore upper-deck SW1xx plant IDs that v84 concatenated into Switch 10038 / 1127 names.
Those are helix and upper-deck motors, not CTC numbers; leave Switch 27/29 and DCC 100–119 alone.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
+++ b/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
@@ -16859,7 +16859,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Switch 1129 N</t>
+          <t>SW129 N</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -16899,7 +16899,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Switch 1129 R</t>
+          <t>SW129 R</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -16939,7 +16939,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Switch 1127 N</t>
+          <t>SW127 N</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -16979,7 +16979,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Switch 1127 R</t>
+          <t>SW127 R</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -17019,7 +17019,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Switch 10038 N</t>
+          <t>SW138 N</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -17059,7 +17059,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Switch 10038 R</t>
+          <t>SW138 R</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -19479,7 +19479,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Switch 1124 N</t>
+          <t>SW124 N</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
@@ -19519,7 +19519,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Switch 1124 R</t>
+          <t>SW124 R</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
@@ -20039,7 +20039,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Switch 10043 N</t>
+          <t>SW143 N</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
@@ -20079,7 +20079,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Switch 10043 R</t>
+          <t>SW143 R</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
@@ -20814,7 +20814,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Switch 10044 N</t>
+          <t>SW144 N</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -20854,7 +20854,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Switch 10044 R</t>
+          <t>SW144 R</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -20894,7 +20894,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Switch 10045 N</t>
+          <t>SW145 N</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -20934,7 +20934,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>Switch 10045 R</t>
+          <t>SW145 R</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
@@ -20974,7 +20974,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Switch 10046 N</t>
+          <t>SW146 N</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
@@ -21014,7 +21014,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Switch 10046 R</t>
+          <t>SW146 R</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
@@ -21054,7 +21054,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>Switch 10047 N</t>
+          <t>SW147 N</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
@@ -21094,7 +21094,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Switch 10047 R</t>
+          <t>SW147 R</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -21699,7 +21699,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>Switch 10048 N</t>
+          <t>SW148 N</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -21739,7 +21739,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>Switch 10048 R</t>
+          <t>SW148 R</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -21779,7 +21779,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Switch 10049 N</t>
+          <t>SW149 N</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -21819,7 +21819,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>Switch 10049 R</t>
+          <t>SW149 R</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -21859,7 +21859,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Switch 10050 N</t>
+          <t>SW150 N</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -21899,7 +21899,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Switch 10050 R</t>
+          <t>SW150 R</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
@@ -26410,7 +26410,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Switch 1129 N FB</t>
+          <t>SW129 N FB</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -26445,7 +26445,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Switch 1129 R FB</t>
+          <t>SW129 R FB</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -26480,7 +26480,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Switch 1127 N FB</t>
+          <t>SW127 N FB</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -26515,7 +26515,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Switch 1127 R FB</t>
+          <t>SW127 R FB</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -26550,7 +26550,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Switch 10038 N FB</t>
+          <t>SW138 N FB</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -26585,7 +26585,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Switch 10038 R FB</t>
+          <t>SW138 R FB</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -26650,7 +26650,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Switch 1129 BTN</t>
+          <t>SW129 BTN</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Switch 1127 BTN</t>
+          <t>SW127 BTN</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -26720,7 +26720,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Switch 10038 BTN</t>
+          <t>SW138 BTN</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -26955,7 +26955,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Switch 1124 N FB</t>
+          <t>SW124 N FB</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -26990,7 +26990,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Switch 1124 R FB</t>
+          <t>SW124 R FB</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -27125,7 +27125,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Switch 1124 BTN</t>
+          <t>SW124 BTN</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -27320,7 +27320,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Switch 10043 N FB</t>
+          <t>SW143 N FB</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -27355,7 +27355,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Switch 10043 R FB</t>
+          <t>SW143 R FB</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -27460,7 +27460,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Switch 10043 BTN</t>
+          <t>SW143 BTN</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -27495,7 +27495,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Switch 10044 N FB</t>
+          <t>SW144 N FB</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -27530,7 +27530,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Switch 10044 R FB</t>
+          <t>SW144 R FB</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -27565,7 +27565,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Switch 10045 N FB</t>
+          <t>SW145 N FB</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -27600,7 +27600,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Switch 10045 R FB</t>
+          <t>SW145 R FB</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -27635,7 +27635,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Switch 10046 N FB</t>
+          <t>SW146 N FB</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -27670,7 +27670,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Switch 10046 R FB</t>
+          <t>SW146 R FB</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -27705,7 +27705,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Switch 10047 N FB</t>
+          <t>SW147 N FB</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -27740,7 +27740,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Switch 10047 R FB</t>
+          <t>SW147 R FB</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -27775,7 +27775,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Switch 10044 BTN</t>
+          <t>SW144 BTN</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -27810,7 +27810,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Switch 10045 BTN</t>
+          <t>SW145 BTN</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -27845,7 +27845,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Switch 10046 BTN</t>
+          <t>SW146 BTN</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -27880,7 +27880,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Switch 10047 BTN</t>
+          <t>SW147 BTN</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -27995,7 +27995,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Switch 10048 N FB</t>
+          <t>SW148 N FB</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -28030,7 +28030,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Switch 10048 R FB</t>
+          <t>SW148 R FB</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -28065,7 +28065,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Switch 10049 N FB</t>
+          <t>SW149 N FB</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -28100,7 +28100,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Switch 10049 R FB</t>
+          <t>SW149 R FB</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -28135,7 +28135,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Switch 10050 N FB</t>
+          <t>SW150 N FB</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -28170,7 +28170,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Switch 10050 R FB</t>
+          <t>SW150 R FB</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -28245,7 +28245,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Switch 10048 BTN</t>
+          <t>SW148 BTN</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -28280,7 +28280,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Switch 10049 BTN</t>
+          <t>SW149 BTN</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -28315,7 +28315,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Switch 10050 BTN</t>
+          <t>SW150 BTN</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -29241,7 +29241,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Switch 1127</t>
+          <t>SW127</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -29318,7 +29318,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Switch 1129</t>
+          <t>SW129</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -29375,7 +29375,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Switch 10038</t>
+          <t>SW138</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -29728,7 +29728,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Switch 1125,Switch 1126,139,Switch 10040</t>
+          <t>SW125, SW126, SW139, SW140</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -30267,7 +30267,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Switch 1124</t>
+          <t>SW124</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -30364,7 +30364,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Switch 1121,Switch 1123</t>
+          <t>SW121, SW123</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -30461,7 +30461,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>SW,120,Switch 1122</t>
+          <t>SW120, SW122</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -30774,7 +30774,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Switch 10048</t>
+          <t>SW148</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -30851,7 +30851,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Switch 10049</t>
+          <t>SW149</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -30908,7 +30908,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Switch 10050</t>
+          <t>SW150</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -31213,7 +31213,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Switch 10041,Switch 10042</t>
+          <t>SW141, SW142</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -31290,7 +31290,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Switch 10043</t>
+          <t>SW143</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -31367,7 +31367,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Switch 10044</t>
+          <t>SW144</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -31444,7 +31444,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Switch 10045</t>
+          <t>SW145</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -31501,7 +31501,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Switch 10046</t>
+          <t>SW146</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -31578,7 +31578,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Switch 10047</t>
+          <t>SW147</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">

</xml_diff>

<commit_message>
Put 38LA on C1 leftover pins and show CTC switch numbers in the inventory.
38LA G/Y were on OU4 (easy to read as C11) while OU3-7/8 sat empty; they now sit with R on the 36-board leftovers. 24RB is three pins on C2-OU3. DCC 100–119 labels become Switch 1…39.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
+++ b/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
@@ -4012,7 +4012,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>C2-OU1-7</t>
+          <t>C2-OU3-6</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -4077,14 +4077,14 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G with 24RA; Y on OU3 (OU1-8 is BS cal); R with 24L</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was whole dwarf on leftover OU3 (OU1-8 is BS cal)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>C2-OU3-8</t>
+          <t>C2-OU3-7</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -4149,14 +4149,14 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was G with 24RA; Y on OU3 (OU1-8 is BS cal); R with 24L</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was whole dwarf on leftover OU3 (OU1-8 is BS cal)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>C2-OU2-7</t>
+          <t>C2-OU3-8</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -4221,7 +4221,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was G with 24RA; Y on OU3 (OU1-8 is BS cal); R with 24L</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was whole dwarf on leftover OU3 (OU1-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -7036,7 +7036,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>C1-OU4-7</t>
+          <t>C1-OU3-7</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -7101,14 +7101,14 @@
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp G; was G/Y with 38LB; R spills to 36RA OU2</t>
+          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp G; was leftover trio on 36 boards; 38LB keeps OU4</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>C1-OU4-8</t>
+          <t>C1-OU3-8</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -7173,7 +7173,7 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp Y; was G/Y with 38LB; R spills to 36RA OU2</t>
+          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp Y; was leftover trio on 36 boards; 38LB keeps OU4</t>
         </is>
       </c>
     </row>
@@ -7245,7 +7245,7 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp R; was G/Y with 38LB; R spills to 36RA OU2</t>
+          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp R; was leftover trio on 36 boards; 38LB keeps OU4</t>
         </is>
       </c>
     </row>
@@ -8956,7 +8956,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>C2-OU1-7 C2-OU3-8 C2-OU2-7</t>
+          <t>C2-OU3-6 C2-OU3-7 C2-OU3-8</t>
         </is>
       </c>
     </row>
@@ -9372,7 +9372,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>C1-OU4-7 C1-OU4-8 C1-OU2-7</t>
+          <t>C1-OU3-7 C1-OU3-8 C1-OU2-7</t>
         </is>
       </c>
     </row>
@@ -9928,7 +9928,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Switch 113, Switch 114, Switch 115</t>
+          <t>Switch 35, Switch 37, Switch 39</t>
         </is>
       </c>
       <c r="P3" t="n">
@@ -9948,12 +9948,12 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>SCXB BTN, SW17 BTN, SW18 BTN</t>
+          <t>Switch 35 BTN, Switch 37 BTN, Switch 39 BTN</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>SCXB N FB, SCXB R FB, SW17 N FB, SW17 R FB, SW18 N FB, SW18 R FB</t>
+          <t>Switch 35 N FB, Switch 35 R FB, Switch 37 N FB, Switch 37 R FB, Switch 39 N FB, Switch 39 R FB</t>
         </is>
       </c>
       <c r="W3" t="n">
@@ -9973,7 +9973,7 @@
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>S1-1, S1-2, S1-3, S1-4</t>
+          <t>36RA, 38LA, 36RB, 38LB</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
@@ -9991,7 +9991,7 @@
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>East Lead, McKees Rocks, McKeesport, Switch 113a, Switch 113b, Switch 114, Switch 115, West Main Ext</t>
+          <t>East Lead, McKees Rocks, McKeesport, Switch 35a, Switch 35b, Switch 37, Switch 39, West Main Ext</t>
         </is>
       </c>
     </row>
@@ -10064,12 +10064,12 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>SW10 BTN, SW11 BTN, SW8 BTN, SW9 BTN</t>
+          <t>Switch 25 BTN, Switch 27 BTN, Switch 29 BTN, Switch 31 BTN</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>SW10 N FB, SW10 R FB, SW11 N FB, SW11 R FB, SW8 N FB, SW8 R FB, SW9 N FB, SW9 R FB</t>
+          <t>Switch 25 N FB, Switch 25 R FB, Switch 27 N FB, Switch 27 R FB, Switch 29 N FB, Switch 29 R FB, Switch 31 N FB, Switch 31 R FB</t>
         </is>
       </c>
       <c r="W4" t="n">
@@ -10089,7 +10089,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>S2-3, S2-5, S2-6, S2-7</t>
+          <t>24RA, 24L, S2-6, S2-7, 24RB</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -10132,7 +10132,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>West - Lower (103–106 motors)</t>
+          <t>West - Lower (Switch 15–21 motors)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -10175,7 +10175,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Switch 103, Switch 104, Switch 105, Switch 106</t>
+          <t>Switch 15, Switch 17, Switch 19, Switch 21</t>
         </is>
       </c>
       <c r="P5" t="n">
@@ -10195,12 +10195,12 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>SW4 BTN, SW5 BTN, SW6 BTN, SW7 BTN</t>
+          <t>Switch 15 BTN, Switch 17 BTN, Switch 19 BTN, Switch 21 BTN</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>SW4 N FB, SW4 R FB, SW5 N FB, SW5 R FB, SW6 N FB, SW6 R FB, SW7 N FB, SW7 R FB</t>
+          <t>Switch 15 N FB, Switch 15 R FB, Switch 17 N FB, Switch 17 R FB, Switch 19 N FB, Switch 19 R FB, Switch 21 N FB, Switch 21 R FB</t>
         </is>
       </c>
       <c r="W5" t="n">
@@ -10220,7 +10220,7 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>S3-11, S3-6, S3-7, S3-8, S3-9</t>
+          <t>S3-6, S3-7, S3-11, S3-8, S3-9</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -10238,12 +10238,12 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>Switch 103, Switch 104, Switch 105, Switch 106, Switch 116</t>
+          <t>Switch 15, Switch 17, Switch 19, Switch 21, Switch 13</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>SW4, SW5, SW6, SW7</t>
+          <t>Switch 15, Switch 17, Switch 19, Switch 21</t>
         </is>
       </c>
     </row>
@@ -10306,7 +10306,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Switch 100, Switch 101, Switch 102, Switch 116</t>
+          <t>Switch 1, Switch 3, Switch 5, Switch 13</t>
         </is>
       </c>
       <c r="P6" t="n">
@@ -10326,12 +10326,12 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>SW1 BTN, SW2 BTN, SW3 BTN</t>
+          <t>Switch 1 BTN, Switch 3 BTN, Switch 5 BTN, Switch 13 BTN</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>SW1 N FB, SW1 R FB, SW2 N FB, SW2 R FB, SW3 N FB, SW3 R FB</t>
+          <t>Switch 1 N FB, Switch 1 R FB, Switch 3 N FB, Switch 3 R FB, Switch 5 N FB, Switch 5 R FB, Switch 13 N FB, Switch 13 R FB</t>
         </is>
       </c>
       <c r="W6" t="n">
@@ -10351,7 +10351,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>S3-1, S3-13, S3-2, S3-3</t>
+          <t>6LB, 6LA, 2L, 4RA, 4RB</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -10369,7 +10369,7 @@
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>Block 100-102, East Main Ext, Switch 100, Switch 101, Switch 102, West Yard Track 1, West Yard Track 2, Yard T1</t>
+          <t>Block 100-102, East Main Ext, Switch 1, Switch 3, Switch 5, West Yard Track 1, West Yard Track 2, Yard T1</t>
         </is>
       </c>
     </row>
@@ -10500,7 +10500,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>SW127, SW129, SW138</t>
+          <t>SW129, SW127, SW138</t>
         </is>
       </c>
       <c r="P8" t="n">
@@ -10535,7 +10535,7 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>S1-5, S1-6, S4-6, S4-7</t>
+          <t>40LB, 40LA, 2036, 2035</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
@@ -10568,7 +10568,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>North - Lower (East End 34 + turnouts 107–112)</t>
+          <t>North - Lower (East End 34 + Switch 25–33)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Switch 107, Switch 108, Switch 109, Switch 110, Switch 111, Switch 112</t>
+          <t>Switch 25, Switch 27, Switch 29, Switch 31, Switch 23, Switch 33</t>
         </is>
       </c>
       <c r="P9" t="n">
@@ -10631,12 +10631,12 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>SCXA BTN, SW12 BTN</t>
+          <t>Switch 25 BTN, Switch 27 BTN, Switch 29 BTN, Switch 31 BTN, Switch 23 BTN, Switch 33 BTN</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>SCXA N FB, SCXA R FB, SW12 N FB, SW12 R FB</t>
+          <t>Switch 25 N FB, Switch 25 R FB, Switch 27 N FB, Switch 27 R FB, Switch 29 N FB, Switch 29 R FB, Switch 31 N FB, Switch 31 R FB, Switch 23 N FB, Switch 23 R FB, Switch 33 N FB, Switch 33 R FB</t>
         </is>
       </c>
       <c r="W9" t="n">
@@ -10656,7 +10656,7 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>S2-1, S2-2, S2-4, S2-8, S2-9</t>
+          <t>34L, 32R, 34R</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
@@ -10674,7 +10674,7 @@
       </c>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>Switch 107, Switch 108, Switch 109, Switch 110, Switch 111a, Switch 111b, Switch 112</t>
+          <t>Switch 25, Switch 27, Switch 29, Switch 31, Switch 23a, Switch 23b, Switch 33</t>
         </is>
       </c>
     </row>
@@ -10732,7 +10732,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Switch 117, Switch 118, Switch 119</t>
+          <t>Switch 7, Switch 11, Switch 9</t>
         </is>
       </c>
       <c r="P10" t="n">
@@ -10750,6 +10750,16 @@
       <c r="T10" t="n">
         <v>0</v>
       </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Switch 7 BTN, Switch 11 BTN, Switch 9 BTN</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Switch 7 N FB, Switch 7 R FB, Switch 11 N FB, Switch 11 R FB, Switch 9 N FB, Switch 9 R FB</t>
+        </is>
+      </c>
       <c r="W10" t="n">
         <v>24</v>
       </c>
@@ -10767,7 +10777,7 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>S3-10, S3-12, S3-14, S3-4, S3-5</t>
+          <t>8RA, S3-14, 8LA, 8LB, 8RB</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
@@ -10780,7 +10790,7 @@
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>Switch 117 (TO6), Switch 117 (TO8), Switch 118, Switch 119, Yard T10, Yard T11, Yard T6, Yard T9</t>
+          <t>Switch 7 (TO6), Switch 7 (TO8), Switch 11, Switch 9, Yard T10, Yard T11, Yard T6, Yard T9</t>
         </is>
       </c>
     </row>
@@ -10888,7 +10898,7 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>S6-1, S6-11, S6-13, S6-2, S6-5</t>
+          <t>S6-2, S6-13, S6-11, S6-1, S6-5</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
@@ -10989,12 +10999,12 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>NIX BTN, SW127 BTN, SW129 BTN, SW138 BTN</t>
+          <t>NIX BTN, SW129 BTN, SW127 BTN, SW138 BTN</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>NIX N FB, NIX R FB, SW127 N FB, SW127 R FB, SW129 N FB, SW129 R FB, SW138 N FB, SW138 R FB</t>
+          <t>NIX N FB, NIX R FB, SW129 N FB, SW129 R FB, SW127 N FB, SW127 R FB, SW138 N FB, SW138 R FB</t>
         </is>
       </c>
       <c r="W12" t="n">
@@ -11014,7 +11024,7 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>S4-1, S4-2, S4-3, S4-4, S4-5</t>
+          <t>S4-1, S4-2, S4-5, S4-3, S4-4</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
@@ -11140,7 +11150,7 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>S5-1, S5-2, S5-3, S5-4, S5-5</t>
+          <t>S5-1, S5-2, S5-5, S5-3, S5-4</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
@@ -11266,7 +11276,7 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>S6-12, S6-14, S6-15, S6-6, S6-8</t>
+          <t>S6-6, S6-8, S6-12, S6-15, S6-14</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
@@ -11392,7 +11402,7 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>S6-10, S6-3, S6-4, S6-7, S6-9</t>
+          <t>S6-10, S6-3, S6-9, S6-4, S6-7</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
@@ -11599,7 +11609,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Switch 113 N</t>
+          <t>Switch 35 N</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -11639,7 +11649,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Switch 113 R</t>
+          <t>Switch 35 R</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -11679,7 +11689,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Switch 114 N</t>
+          <t>Switch 37 N</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -11719,7 +11729,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Switch 114 R</t>
+          <t>Switch 37 R</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -11759,7 +11769,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Switch 115 N</t>
+          <t>Switch 39 N</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -11799,7 +11809,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Switch 115 R</t>
+          <t>Switch 39 R</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -12461,15 +12471,30 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Helix - Lower</t>
+          <t>Helix - Lower (Princess SW37)</t>
         </is>
       </c>
       <c r="D24" t="n">
         <v>7</v>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Head 38LA G</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Searchlight Signal Head</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/143; packed 143 (node 1 sig 11)</t>
         </is>
       </c>
     </row>
@@ -12486,15 +12511,30 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Helix - Lower</t>
+          <t>Helix - Lower (Princess SW37)</t>
         </is>
       </c>
       <c r="D25" t="n">
         <v>8</v>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Head 38LA Y</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Searchlight Signal Head</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/143; packed 143 (node 1 sig 11)</t>
         </is>
       </c>
     </row>
@@ -12519,7 +12559,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Switch 107 N</t>
+          <t>Switch 25 N</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -12559,7 +12599,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Switch 107 R</t>
+          <t>Switch 25 R</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -12599,7 +12639,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Switch 108 N</t>
+          <t>Switch 27 N</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -12639,7 +12679,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Switch 108 R</t>
+          <t>Switch 27 R</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -12679,7 +12719,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Switch 109 N</t>
+          <t>Switch 29 N</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -12719,7 +12759,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Switch 109 R</t>
+          <t>Switch 29 R</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -12759,7 +12799,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Switch 110 N</t>
+          <t>Switch 31 N</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -12799,7 +12839,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Switch 110 R</t>
+          <t>Switch 31 R</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -13711,30 +13751,20 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>North - Lower (East End west 24)</t>
+          <t>North - Lower</t>
         </is>
       </c>
       <c r="D56" t="n">
         <v>7</v>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Head 24RB G</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Searchlight Signal Head</t>
-        </is>
-      </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
+          <t>free — linear6 turnouts on radio addr 12 live on C12 (C2 radio addr is 2; block sensors only)</t>
         </is>
       </c>
     </row>
@@ -14031,7 +14061,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>North - Lower (East End west 24)</t>
+          <t>North - Lower</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -14039,22 +14069,17 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Head 24RB R</t>
+          <t>S2-6 Y</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Dwarf Upgrade</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
           <t>5V</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/234; packed 234 (node 2 sig 2); was S2-6 Y</t>
         </is>
       </c>
     </row>
@@ -14281,15 +14306,30 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>North - Lower</t>
+          <t>North - Lower (East End west 24)</t>
         </is>
       </c>
       <c r="D71" t="n">
         <v>6</v>
       </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Head 24RB G</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Searchlight Signal Head</t>
+        </is>
+      </c>
       <c r="G71" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
         </is>
       </c>
     </row>
@@ -14306,15 +14346,30 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>North - Lower</t>
+          <t>North - Lower (East End west 24)</t>
         </is>
       </c>
       <c r="D72" t="n">
         <v>7</v>
       </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Head 24RB Y</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Searchlight Signal Head</t>
+        </is>
+      </c>
       <c r="G72" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
         </is>
       </c>
     </row>
@@ -14339,7 +14394,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Head 24RB Y</t>
+          <t>Head 24RB R</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -14354,7 +14409,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
         </is>
       </c>
     </row>
@@ -14379,7 +14434,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Switch 103 N</t>
+          <t>Switch 15 N</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -14419,7 +14474,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Switch 103 R</t>
+          <t>Switch 15 R</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -14459,7 +14514,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Switch 104 N</t>
+          <t>Switch 17 N</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -14499,7 +14554,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Switch 104 R</t>
+          <t>Switch 17 R</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -14539,7 +14594,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Switch 105 N</t>
+          <t>Switch 19 N</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -14579,7 +14634,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Switch 105 R</t>
+          <t>Switch 19 R</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -14619,7 +14674,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Switch 106 N</t>
+          <t>Switch 21 N</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -14659,7 +14714,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Switch 106 R</t>
+          <t>Switch 21 R</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -15899,7 +15954,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Switch 100 N</t>
+          <t>Switch 1 N</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -15939,7 +15994,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Switch 100 R</t>
+          <t>Switch 1 R</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -15979,7 +16034,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Switch 101 N</t>
+          <t>Switch 3 N</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -16019,7 +16074,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Switch 101 R</t>
+          <t>Switch 3 R</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -16059,7 +16114,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Switch 102 N</t>
+          <t>Switch 5 N</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -16099,7 +16154,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Switch 102 R</t>
+          <t>Switch 5 R</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -16139,7 +16194,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Switch 116 N</t>
+          <t>Switch 13 N</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -16179,7 +16234,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Switch 116 R</t>
+          <t>Switch 13 R</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -22554,7 +22609,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Switch 117 N</t>
+          <t>Switch 7 N</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
@@ -22594,7 +22649,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Switch 117 R</t>
+          <t>Switch 7 R</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
@@ -22634,7 +22689,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Switch 118 N</t>
+          <t>Switch 11 N</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
@@ -22674,7 +22729,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Switch 118 R</t>
+          <t>Switch 11 R</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
@@ -22714,7 +22769,7 @@
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>Switch 119 N</t>
+          <t>Switch 9 N</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
@@ -22754,7 +22809,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Switch 119 R</t>
+          <t>Switch 9 R</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
@@ -22854,7 +22909,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>Switch 111 N</t>
+          <t>Switch 23 N</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
@@ -22894,7 +22949,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Switch 111 R</t>
+          <t>Switch 23 R</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
@@ -22934,7 +22989,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Switch 112 N</t>
+          <t>Switch 33 N</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
@@ -22974,7 +23029,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Switch 112 R</t>
+          <t>Switch 33 R</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
@@ -23366,22 +23421,12 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Helix - Lower (Princess SW37)</t>
+          <t>Helix - Lower</t>
         </is>
       </c>
       <c r="D320" t="n">
         <v>7</v>
       </c>
-      <c r="E320" t="inlineStr">
-        <is>
-          <t>Head 38LA G</t>
-        </is>
-      </c>
-      <c r="F320" t="inlineStr">
-        <is>
-          <t>Searchlight Signal Head</t>
-        </is>
-      </c>
       <c r="G320" t="inlineStr">
         <is>
           <t>5V</t>
@@ -23389,7 +23434,7 @@
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/143; packed 143 (node 1 sig 11)</t>
+          <t>NEW 5V DNOU8 (OU4) for second searchlight disc</t>
         </is>
       </c>
     </row>
@@ -23406,22 +23451,12 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>Helix - Lower (Princess SW37)</t>
+          <t>Helix - Lower</t>
         </is>
       </c>
       <c r="D321" t="n">
         <v>8</v>
       </c>
-      <c r="E321" t="inlineStr">
-        <is>
-          <t>Head 38LA Y</t>
-        </is>
-      </c>
-      <c r="F321" t="inlineStr">
-        <is>
-          <t>Searchlight Signal Head</t>
-        </is>
-      </c>
       <c r="G321" t="inlineStr">
         <is>
           <t>5V</t>
@@ -23429,7 +23464,7 @@
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/143; packed 143 (node 1 sig 11)</t>
+          <t>NEW 5V DNOU8 (OU4) for second searchlight disc</t>
         </is>
       </c>
     </row>
@@ -24120,7 +24155,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Switch 113 N FB</t>
+          <t>Switch 35 N FB</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -24155,7 +24190,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Switch 113 R FB</t>
+          <t>Switch 35 R FB</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -24190,7 +24225,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Switch 114 N FB</t>
+          <t>Switch 37 N FB</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -24225,7 +24260,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Switch 114 R FB</t>
+          <t>Switch 37 R FB</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -24260,7 +24295,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Switch 115 N FB</t>
+          <t>Switch 39 N FB</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -24295,7 +24330,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Switch 115 R FB</t>
+          <t>Switch 39 R FB</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -24370,7 +24405,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Switch 113 BTN</t>
+          <t>Switch 35 BTN</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -24405,7 +24440,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Switch 114 BTN</t>
+          <t>Switch 37 BTN</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -24440,7 +24475,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Switch 115 BTN</t>
+          <t>Switch 39 BTN</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -24575,7 +24610,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Switch 107 N FB</t>
+          <t>Switch 25 N FB</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -24610,7 +24645,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Switch 107 R FB</t>
+          <t>Switch 25 R FB</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -24645,7 +24680,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Switch 108 N FB</t>
+          <t>Switch 27 N FB</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -24680,7 +24715,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Switch 108 R FB</t>
+          <t>Switch 27 R FB</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -24715,7 +24750,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Switch 109 N FB</t>
+          <t>Switch 29 N FB</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -24750,7 +24785,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Switch 109 R FB</t>
+          <t>Switch 29 R FB</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -24785,7 +24820,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Switch 110 N FB</t>
+          <t>Switch 31 N FB</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -24820,7 +24855,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Switch 110 R FB</t>
+          <t>Switch 31 R FB</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -24855,7 +24890,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Switch 107 N FB</t>
+          <t>Switch 25 N FB</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -24890,7 +24925,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Switch 107 R FB</t>
+          <t>Switch 25 R FB</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -24925,7 +24960,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Switch 108 N FB</t>
+          <t>Switch 27 N FB</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -24960,7 +24995,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Switch 108 R FB</t>
+          <t>Switch 27 R FB</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -24995,7 +25030,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Switch 109 N FB</t>
+          <t>Switch 29 N FB</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -25030,7 +25065,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Switch 109 R FB</t>
+          <t>Switch 29 R FB</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -25065,7 +25100,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Switch 110 N FB</t>
+          <t>Switch 31 N FB</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -25100,7 +25135,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Switch 110 R FB</t>
+          <t>Switch 31 R FB</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -25135,7 +25170,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Switch 107 BTN</t>
+          <t>Switch 25 BTN</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -25170,7 +25205,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Switch 108 BTN</t>
+          <t>Switch 27 BTN</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -25205,7 +25240,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Switch 109 BTN</t>
+          <t>Switch 29 BTN</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -25240,7 +25275,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Switch 110 BTN</t>
+          <t>Switch 31 BTN</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -25355,7 +25390,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Switch 103 N FB</t>
+          <t>Switch 15 N FB</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -25390,7 +25425,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Switch 103 R FB</t>
+          <t>Switch 15 R FB</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -25425,7 +25460,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Switch 104 N FB</t>
+          <t>Switch 17 N FB</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -25460,7 +25495,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Switch 104 R FB</t>
+          <t>Switch 17 R FB</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -25495,7 +25530,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Switch 105 N FB</t>
+          <t>Switch 19 N FB</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -25530,7 +25565,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Switch 105 R FB</t>
+          <t>Switch 19 R FB</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -25565,7 +25600,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Switch 106 N FB</t>
+          <t>Switch 21 N FB</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -25600,7 +25635,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Switch 106 R FB</t>
+          <t>Switch 21 R FB</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -25635,7 +25670,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Switch 103 BTN</t>
+          <t>Switch 15 BTN</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -25670,7 +25705,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Switch 104 BTN</t>
+          <t>Switch 17 BTN</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -25705,7 +25740,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Switch 105 BTN</t>
+          <t>Switch 19 BTN</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -25740,7 +25775,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Switch 106 BTN</t>
+          <t>Switch 21 BTN</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -25855,7 +25890,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Switch 100 N FB</t>
+          <t>Switch 1 N FB</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -25890,7 +25925,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Switch 100 R FB</t>
+          <t>Switch 1 R FB</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -25925,7 +25960,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Switch 101 N FB</t>
+          <t>Switch 3 N FB</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -25960,7 +25995,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Switch 101 R FB</t>
+          <t>Switch 3 R FB</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -25995,7 +26030,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Switch 102 N FB</t>
+          <t>Switch 5 N FB</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -26030,7 +26065,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Switch 102 R FB</t>
+          <t>Switch 5 R FB</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -26065,7 +26100,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Switch 116 N FB</t>
+          <t>Switch 13 N FB</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -26100,7 +26135,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Switch 116 R FB</t>
+          <t>Switch 13 R FB</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -26135,7 +26170,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Switch 100 BTN</t>
+          <t>Switch 1 BTN</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -26170,7 +26205,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Switch 101 BTN</t>
+          <t>Switch 3 BTN</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -26205,7 +26240,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Switch 102 BTN</t>
+          <t>Switch 5 BTN</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -26240,7 +26275,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Switch 116 BTN</t>
+          <t>Switch 13 BTN</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -28450,7 +28485,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Switch 117 N FB</t>
+          <t>Switch 7 N FB</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -28485,7 +28520,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Switch 117 R FB</t>
+          <t>Switch 7 R FB</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -28520,7 +28555,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Switch 118 N FB</t>
+          <t>Switch 11 N FB</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -28555,7 +28590,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Switch 118 R FB</t>
+          <t>Switch 11 R FB</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -28590,7 +28625,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Switch 119 N FB</t>
+          <t>Switch 9 N FB</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -28625,7 +28660,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Switch 119 R FB</t>
+          <t>Switch 9 R FB</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -28660,7 +28695,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Switch 117 BTN</t>
+          <t>Switch 7 BTN</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -28695,7 +28730,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Switch 118 BTN</t>
+          <t>Switch 11 BTN</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -28730,7 +28765,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Switch 119 BTN</t>
+          <t>Switch 9 BTN</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -28765,7 +28800,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Switch 111 N FB</t>
+          <t>Switch 23 N FB</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -28800,7 +28835,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Switch 111 R FB</t>
+          <t>Switch 23 R FB</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -28835,7 +28870,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Switch 112 N FB</t>
+          <t>Switch 33 N FB</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -28870,7 +28905,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Switch 112 R FB</t>
+          <t>Switch 33 R FB</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -28905,7 +28940,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Switch 107 BTN</t>
+          <t>Switch 25 BTN</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -28940,7 +28975,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Switch 108 BTN</t>
+          <t>Switch 27 BTN</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -28975,7 +29010,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Switch 109 BTN</t>
+          <t>Switch 29 BTN</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -29010,7 +29045,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Switch 110 BTN</t>
+          <t>Switch 31 BTN</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -29045,7 +29080,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Switch 111 BTN</t>
+          <t>Switch 23 BTN</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -29080,7 +29115,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Switch 112 BTN</t>
+          <t>Switch 33 BTN</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -29452,7 +29487,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Switch 113a, Switch 113b (TOL2/TOL1)</t>
+          <t>Switch 35a, Switch 35b (TOL2/TOL1)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -29488,11 +29523,6 @@
       <c r="K5" t="inlineStr">
         <is>
           <t>C1-OU2-1</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>S1-3</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -29549,7 +29579,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Switch 114</t>
+          <t>Switch 37</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -29646,7 +29676,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Switch 115</t>
+          <t>Switch 39</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -29825,7 +29855,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Switch 111a, Switch 111b (TOR31/TOR32)</t>
+          <t>Switch 23a, Switch 23b (TOR31/TOR32)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -29922,7 +29952,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Switch 112</t>
+          <t>Switch 33</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -29984,7 +30014,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Switch 109</t>
+          <t>Switch 29</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -29999,7 +30029,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Switch 109</t>
+          <t>Switch 29</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -30076,7 +30106,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Switch 110</t>
+          <t>Switch 31</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -30112,11 +30142,6 @@
       <c r="K12" t="inlineStr">
         <is>
           <t>C12-OU2-7</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>S2-1</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -30138,7 +30163,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Switch 107</t>
+          <t>Switch 25</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -30153,7 +30178,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Switch 107</t>
+          <t>Switch 25</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -30195,7 +30220,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Switch 108</t>
+          <t>Switch 27</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -30210,7 +30235,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Switch 108</t>
+          <t>Switch 27</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -30538,7 +30563,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Switch 100</t>
+          <t>Switch 1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -30595,7 +30620,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Switch 101</t>
+          <t>Switch 3</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -30611,26 +30636,6 @@
       <c r="G19" t="inlineStr">
         <is>
           <t>C4-IN1-4</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>S1-1</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>C1-OU2-3</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>C1-OU2-2</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>C1-OU2-1</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -30677,7 +30682,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Switch 102</t>
+          <t>Switch 5</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -30713,11 +30718,6 @@
       <c r="K20" t="inlineStr">
         <is>
           <t>C4-OU2-7</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>S3-6</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -30950,7 +30950,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Switch 103</t>
+          <t>Switch 15</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -30965,7 +30965,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Switch 103</t>
+          <t>Switch 15</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -31027,7 +31027,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Switch 104</t>
+          <t>Switch 17</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -31042,7 +31042,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Switch 104</t>
+          <t>Switch 17</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -31084,7 +31084,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Switch 105</t>
+          <t>Switch 19</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -31099,7 +31099,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Switch 105</t>
+          <t>Switch 19</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -31141,7 +31141,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Switch 106</t>
+          <t>Switch 21</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -31156,7 +31156,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Switch 106</t>
+          <t>Switch 21</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -31600,7 +31600,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Switch 116</t>
+          <t>Switch 13</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -31615,7 +31615,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Switch 116 (TO1)</t>
+          <t>Switch 13 (TO1)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -31652,7 +31652,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Switch 117 / TO6+TO8</t>
+          <t>Switch 7 / TO6+TO8</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -31704,7 +31704,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Switch 118</t>
+          <t>Switch 11</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -31719,7 +31719,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Switch 118 (TO11)</t>
+          <t>Switch 11 (TO11)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -31741,7 +31741,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Switch 119</t>
+          <t>Switch 9</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -31756,7 +31756,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Switch 119 (TO10)</t>
+          <t>Switch 9 (TO10)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -31858,7 +31858,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Switch 101</t>
+          <t>Switch 3</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -31903,7 +31903,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Switch 100</t>
+          <t>Switch 1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -32038,7 +32038,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Switch 102</t>
+          <t>Switch 5</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -32133,7 +32133,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>SW2, SW3</t>
+          <t>Switch 3, Switch 5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -32218,7 +32218,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Switch 116</t>
+          <t>Switch 13</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -32263,7 +32263,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Switch 103</t>
+          <t>Switch 15</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -32308,7 +32308,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Switch 104</t>
+          <t>Switch 17</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -32358,7 +32358,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SW5, Yard 2a</t>
+          <t>Switch 17, Yard 2a</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -32398,7 +32398,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Switch 105</t>
+          <t>Switch 19</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -32448,7 +32448,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SW6, Yard 3a</t>
+          <t>Switch 19, Yard 3a</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -32488,7 +32488,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Switch 106</t>
+          <t>Switch 21</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -32538,7 +32538,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>SW7, Yard 4a</t>
+          <t>Switch 21, Yard 4a</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -32938,7 +32938,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Switch 107</t>
+          <t>Switch 25</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -32988,7 +32988,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>SW8, Yard 3a, SW10</t>
+          <t>Switch 25, Yard 3a, Switch 29</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -33028,7 +33028,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Switch 108</t>
+          <t>Switch 27</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -33073,7 +33073,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Switch 111a</t>
+          <t>Switch 23a</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -33118,7 +33118,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Switch 109</t>
+          <t>Switch 29</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -33163,7 +33163,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Switch 111b</t>
+          <t>Switch 23b</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -33208,7 +33208,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Switch 110</t>
+          <t>Switch 31</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -33253,7 +33253,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Switch 112</t>
+          <t>Switch 33</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -33388,7 +33388,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Switch 114</t>
+          <t>Switch 37</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -33433,7 +33433,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Switch 115</t>
+          <t>Switch 39</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -33478,7 +33478,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Switch 113b</t>
+          <t>Switch 35b</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -33523,7 +33523,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Switch 113a</t>
+          <t>Switch 35a</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -33663,7 +33663,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>SW18, Helix Inner B</t>
+          <t>Switch 39, Helix Inner B</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -33703,7 +33703,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>SW17, Helix Outer B</t>
+          <t>Switch 37, Helix Outer B</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -35353,7 +35353,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Switch 118</t>
+          <t>Switch 11</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -35398,7 +35398,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Switch 117 (TO8)</t>
+          <t>Switch 7 (TO8)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -35443,7 +35443,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Switch 117 (TO6)</t>
+          <t>Switch 7 (TO6)</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -35623,7 +35623,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Switch 119</t>
+          <t>Switch 9</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">

</xml_diff>

<commit_message>
Put 40LA on three consecutive C11-OU3 pins; 2035/2036 sit as separate dwarfs.
Refresh the Desktop wiring pack so C1 motors show Switch 35/37/39 instead of DCC 113–115.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
+++ b/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
@@ -7684,7 +7684,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>C11-OU2-7</t>
+          <t>C11-OU3-1</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -7749,14 +7749,14 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was G with 40LB; Y/R on balloon OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was whole dwarf on OU3; 2035/2036 can sit apart</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>C11-OU3-8</t>
+          <t>C11-OU3-2</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -7821,14 +7821,14 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp Y; was G with 40LB; Y/R on balloon OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp Y; was whole dwarf on OU3; 2035/2036 can sit apart</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>C11-OU3-7</t>
+          <t>C11-OU3-3</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -7893,14 +7893,14 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was G with 40LB; Y/R on balloon OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was whole dwarf on OU3; 2035/2036 can sit apart</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>C11-OU3-1</t>
+          <t>C11-OU3-4</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -7965,14 +7965,14 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was S1-6; sequential G/Y/R</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was balloon; sequential G/Y/R</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>C11-OU3-2</t>
+          <t>C11-OU3-5</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -8037,14 +8037,14 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp Y; was S1-6; sequential G/Y/R</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp Y; was balloon; sequential G/Y/R</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>C11-OU3-3</t>
+          <t>C11-OU3-6</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -8109,14 +8109,14 @@
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was S1-6; sequential G/Y/R</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was balloon; sequential G/Y/R</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>C11-OU3-4</t>
+          <t>C11-OU3-7</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -8181,14 +8181,14 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was S4-6; sequential G/Y/R</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was leftover trio (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>C11-OU3-5</t>
+          <t>C11-OU3-8</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -8253,14 +8253,14 @@
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was S4-6; sequential G/Y/R</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was leftover trio (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>C11-OU3-6</t>
+          <t>C11-OU2-7</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was S4-6; sequential G/Y/R</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was leftover trio (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -9476,7 +9476,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>C11-OU2-7 C11-OU3-8 C11-OU3-7</t>
+          <t>C11-OU3-1 C11-OU3-2 C11-OU3-3</t>
         </is>
       </c>
     </row>
@@ -9528,7 +9528,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>C11-OU3-1 C11-OU3-2 C11-OU3-3</t>
+          <t>C11-OU3-4 C11-OU3-5 C11-OU3-6</t>
         </is>
       </c>
     </row>
@@ -9580,7 +9580,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>C11-OU3-4 C11-OU3-5 C11-OU3-6</t>
+          <t>C11-OU3-7 C11-OU3-8 C11-OU2-7</t>
         </is>
       </c>
     </row>
@@ -10535,7 +10535,7 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>40LB, 40LA, 2036, 2035</t>
+          <t>40LB, 2035, 40LA, 2036</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
@@ -17436,7 +17436,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Helix (Princess east SW39)</t>
+          <t>Helix (balloon 115)</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -17444,7 +17444,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Head 40LA G</t>
+          <t>Head 2035 R</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -17459,7 +17459,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2)</t>
         </is>
       </c>
     </row>
@@ -17516,7 +17516,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Helix (balloon 114)</t>
+          <t>Helix (Princess east SW39)</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -17524,7 +17524,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Head 2036 G</t>
+          <t>Head 40LA G</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -17539,7 +17539,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-6 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4); was S4-6 G</t>
         </is>
       </c>
     </row>
@@ -17556,7 +17556,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Helix (balloon 114)</t>
+          <t>Helix (Princess east SW39)</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -17564,7 +17564,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Head 2036 Y</t>
+          <t>Head 40LA Y</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -17579,7 +17579,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-6 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4); was S4-6 R</t>
         </is>
       </c>
     </row>
@@ -17596,7 +17596,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Helix (balloon 114)</t>
+          <t>Helix (Princess east SW39)</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -17604,7 +17604,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Head 2036 R</t>
+          <t>Head 40LA R</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -17619,7 +17619,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-6 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4); was S4-6 Y</t>
         </is>
       </c>
     </row>
@@ -17636,7 +17636,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Helix (balloon 115)</t>
+          <t>Helix (balloon 114)</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -17644,7 +17644,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Head 2035 G</t>
+          <t>Head 2036 G</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -17659,7 +17659,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2); was S4-7 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-7 G</t>
         </is>
       </c>
     </row>
@@ -17676,7 +17676,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Helix (balloon 115)</t>
+          <t>Helix (balloon 114)</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -17684,7 +17684,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Head 2035 Y</t>
+          <t>Head 2036 Y</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -17699,7 +17699,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2); was S4-7 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-7 R</t>
         </is>
       </c>
     </row>
@@ -17716,7 +17716,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Helix (balloon 115)</t>
+          <t>Helix (balloon 114)</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -17724,7 +17724,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Head 2035 R</t>
+          <t>Head 2036 R</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -17739,7 +17739,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2); was S4-7 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-7 Y</t>
         </is>
       </c>
     </row>
@@ -17756,7 +17756,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Helix (Princess east SW39)</t>
+          <t>Helix (balloon 115)</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -17764,7 +17764,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Head 40LA R</t>
+          <t>Head 2035 G</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -17779,7 +17779,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2)</t>
         </is>
       </c>
     </row>
@@ -17796,7 +17796,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Helix (Princess east SW39)</t>
+          <t>Helix (balloon 115)</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -17804,7 +17804,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Head 40LA Y</t>
+          <t>Head 2035 Y</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -17819,7 +17819,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2)</t>
         </is>
       </c>
     </row>
@@ -29604,17 +29604,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>C11-OU3-3</t>
+          <t>C11-OU3-6</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>C11-OU3-2</t>
+          <t>C11-OU3-5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>C11-OU3-1</t>
+          <t>C11-OU3-4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -29701,17 +29701,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>C11-OU3-6</t>
+          <t>C11-OU2-7</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>C11-OU3-5</t>
+          <t>C11-OU3-8</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>C11-OU3-4</t>
+          <t>C11-OU3-7</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">

</xml_diff>

<commit_message>
Number upper-deck plants from Switch 61 / 62L and drop leftover C2 S2 RGB.
Same odd-switch even-signal pattern as the lower deck. C2-OU3 stays because 24RB still needs three pins.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
+++ b/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
@@ -10089,7 +10089,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>24RA, 24L, S2-6, S2-7, 24RB</t>
+          <t>24RA, 24L, 24RB</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -10495,7 +10495,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>SW129, SW127, SW138</t>
+          <t>Switch 67, Switch 63, Switch 65</t>
         </is>
       </c>
       <c r="P8" t="n">
@@ -10848,7 +10848,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>SW144, SW145, SW146, SW147</t>
+          <t>Switch 79, Switch 81, Switch 83, Switch 85</t>
         </is>
       </c>
       <c r="P11" t="n">
@@ -10868,12 +10868,12 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>SW144 BTN, SW145 BTN, SW146 BTN, SW147 BTN</t>
+          <t>Switch 79 BTN, Switch 81 BTN, Switch 83 BTN, Switch 85 BTN</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>SW144 N FB, SW144 R FB, SW145 N FB, SW145 R FB, SW146 N FB, SW146 R FB, SW147 N FB, SW147 R FB</t>
+          <t>Switch 79 N FB, Switch 79 R FB, Switch 81 N FB, Switch 81 R FB, Switch 83 N FB, Switch 83 R FB, Switch 85 N FB, Switch 85 R FB</t>
         </is>
       </c>
       <c r="W11" t="n">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>S6-2, S6-13, S6-11, S6-1, S6-5</t>
+          <t>76R, 86L, 84RA, 76L, 78RB</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>PTT1, PTT2, SW143, SW144, SW145, SW146, SW147, TT</t>
+          <t>PTT1, PTT2, Switch 77, Switch 79, Switch 81, Switch 83, Switch 85, TT</t>
         </is>
       </c>
     </row>
@@ -10974,7 +10974,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>NIX</t>
+          <t>Switch 61</t>
         </is>
       </c>
       <c r="P12" t="n">
@@ -10994,12 +10994,12 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>NIX BTN, SW129 BTN, SW127 BTN, SW138 BTN</t>
+          <t>Switch 61 BTN, Switch 67 BTN, Switch 63 BTN, Switch 65 BTN</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>NIX N FB, NIX R FB, SW129 N FB, SW129 R FB, SW127 N FB, SW127 R FB, SW138 N FB, SW138 R FB</t>
+          <t>Switch 61 N FB, Switch 61 R FB, Switch 67 N FB, Switch 67 R FB, Switch 63 N FB, Switch 63 R FB, Switch 65 N FB, Switch 65 R FB</t>
         </is>
       </c>
       <c r="W12" t="n">
@@ -11019,7 +11019,7 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>S4-1, S4-2, S4-5, S4-3, S4-4</t>
+          <t>64R, 68L, 66RB, 64L, 66RA</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
@@ -11037,7 +11037,7 @@
       </c>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>NIL A, NIL B, Outer Leg, SW125,126, SW127, SW129, SW138, SW139,140</t>
+          <t>NIL A, NIL B, Outer Leg, Switch 61a,126, Switch 63, Switch 67, Switch 65, Switch 61c,140</t>
         </is>
       </c>
     </row>
@@ -11100,7 +11100,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>DJE, DJW</t>
+          <t>Switch 69, Switch 71</t>
         </is>
       </c>
       <c r="P13" t="n">
@@ -11120,12 +11120,12 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>DJE BTN, DJW BTN, SW124 BTN</t>
+          <t>Switch 69 BTN, Switch 71 BTN, Switch 73 BTN</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>DJE N FB, DJE R FB, DJW N FB, DJW R FB, SW124 N FB, SW124 R FB</t>
+          <t>Switch 69 N FB, Switch 69 R FB, Switch 71 N FB, Switch 71 R FB, Switch 73 N FB, Switch 73 R FB</t>
         </is>
       </c>
       <c r="W13" t="n">
@@ -11145,7 +11145,7 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>S5-1, S5-2, S5-5, S5-3, S5-4</t>
+          <t>70L, 72L, 70RA, 74L, 74RA</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
@@ -11163,7 +11163,7 @@
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>Closet Inner, Closet Outer, Outside Inner A, Outside Outer A, SW120, SW121, SW122,123, SW124</t>
+          <t>Closet Inner, Closet Outer, Outside Inner A, Outside Outer A, Switch 71a, Switch 69a, Switch 71b,123, Switch 73</t>
         </is>
       </c>
     </row>
@@ -11226,7 +11226,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>CBX, SW143</t>
+          <t>Switch 75, Switch 77</t>
         </is>
       </c>
       <c r="P14" t="n">
@@ -11246,12 +11246,12 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>CBX BTN, SW143 BTN</t>
+          <t>Switch 75 BTN, Switch 77 BTN</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>CBX N FB, CBX R FB, SW143 N FB, SW143 R FB</t>
+          <t>Switch 75 N FB, Switch 75 R FB, Switch 77 N FB, Switch 77 R FB</t>
         </is>
       </c>
       <c r="W14" t="n">
@@ -11271,7 +11271,7 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>S6-6, S6-8, S6-12, S6-15, S6-14</t>
+          <t>78R, 88R, 84RB, 92L, 90L</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
@@ -11289,7 +11289,7 @@
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>CB Inner A, CB Inner B, CB Outer A, CB Outer B, Outside Inner B, Outside Outer B, SW141, SW142</t>
+          <t>CB Inner A, CB Inner B, CB Outer A, CB Outer B, Outside Inner B, Outside Outer B, Switch 75a, Switch 75b</t>
         </is>
       </c>
     </row>
@@ -11352,7 +11352,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>SW148, SW149, SW150</t>
+          <t>Switch 87, Switch 89, Switch 91</t>
         </is>
       </c>
       <c r="P15" t="n">
@@ -11372,12 +11372,12 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>SW148 BTN, SW149 BTN, SW150 BTN</t>
+          <t>Switch 87 BTN, Switch 89 BTN, Switch 91 BTN</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>SW148 N FB, SW148 R FB, SW149 N FB, SW149 R FB, SW150 N FB, SW150 R FB</t>
+          <t>Switch 87 N FB, Switch 87 R FB, Switch 89 N FB, Switch 89 R FB, Switch 91 N FB, Switch 91 R FB</t>
         </is>
       </c>
       <c r="W15" t="n">
@@ -11397,7 +11397,7 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>S6-10, S6-3, S6-9, S6-4, S6-7</t>
+          <t>82L, 78L, 88RA, 78RA, 88L</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
@@ -11415,7 +11415,7 @@
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>BW1, BW2, CB Siding, CB Station, SW148, SW149, SW150, WH</t>
+          <t>BW1, BW2, CB Siding, CB Station, Switch 87, Switch 89, Switch 91, WH</t>
         </is>
       </c>
     </row>
@@ -11473,7 +11473,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>SW124</t>
+          <t>Switch 73</t>
         </is>
       </c>
       <c r="P16" t="n">
@@ -11508,7 +11508,7 @@
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>S5-6, S5-7</t>
+          <t>70RB, 74RB</t>
         </is>
       </c>
       <c r="AE16" t="n">
@@ -14062,19 +14062,14 @@
       <c r="D64" t="n">
         <v>7</v>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>S2-6 Y</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Dwarf Upgrade</t>
-        </is>
-      </c>
       <c r="G64" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>spare (CP2 leftover RGB removed; was S2-6 Y)</t>
         </is>
       </c>
     </row>
@@ -14132,19 +14127,14 @@
       <c r="D66" t="n">
         <v>1</v>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>S2-6 G</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Signal LED</t>
-        </is>
-      </c>
       <c r="G66" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>spare (CP2 leftover RGB removed; was S2-6 G)</t>
         </is>
       </c>
     </row>
@@ -14167,19 +14157,14 @@
       <c r="D67" t="n">
         <v>2</v>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>S2-6 R</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Signal LED</t>
-        </is>
-      </c>
       <c r="G67" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>spare (CP2 leftover RGB removed; was S2-6 R)</t>
         </is>
       </c>
     </row>
@@ -14202,19 +14187,14 @@
       <c r="D68" t="n">
         <v>3</v>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>S2-7 G</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>Signal LED</t>
-        </is>
-      </c>
       <c r="G68" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>spare (CP2 leftover RGB removed; was S2-7 G)</t>
         </is>
       </c>
     </row>
@@ -14237,19 +14217,14 @@
       <c r="D69" t="n">
         <v>4</v>
       </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>S2-7 R</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>Signal LED</t>
-        </is>
-      </c>
       <c r="G69" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>spare (CP2 leftover RGB removed; was S2-7 R)</t>
         </is>
       </c>
     </row>
@@ -14272,19 +14247,14 @@
       <c r="D70" t="n">
         <v>5</v>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>S2-7 Y</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>Dwarf Upgrade</t>
-        </is>
-      </c>
       <c r="G70" t="inlineStr">
         <is>
           <t>5V</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>spare (CP2 leftover RGB removed; was S2-7 Y)</t>
         </is>
       </c>
     </row>
@@ -16589,7 +16559,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>SW129 N</t>
+          <t>Switch 67 N</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -16629,7 +16599,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>SW129 R</t>
+          <t>Switch 67 R</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -16669,7 +16639,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>SW127 N</t>
+          <t>Switch 63 N</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -16709,7 +16679,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>SW127 R</t>
+          <t>Switch 63 R</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -16749,7 +16719,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>SW138 N</t>
+          <t>Switch 65 N</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -16789,7 +16759,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>SW138 R</t>
+          <t>Switch 65 R</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -17519,7 +17489,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>NIX N</t>
+          <t>Switch 61 N</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -17554,7 +17524,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>NIX R</t>
+          <t>Switch 61 R</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -17799,7 +17769,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Head S4-1 G</t>
+          <t>Head 64R G</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -17814,7 +17784,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>CP4 | Closet Outer → Aristech | Closet Outer | defined head</t>
+          <t>CP4 | Closet Outer → Aristech | Closet Outer | defined head | was S4-1</t>
         </is>
       </c>
     </row>
@@ -17839,7 +17809,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Head S4-1 Y</t>
+          <t>Head 64R Y</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -17854,7 +17824,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>CP4 | Closet Outer → Aristech | Closet Outer | defined head</t>
+          <t>CP4 | Closet Outer → Aristech | Closet Outer | defined head | was S4-1</t>
         </is>
       </c>
     </row>
@@ -17879,7 +17849,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Head S4-1 R</t>
+          <t>Head 64R R</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -17894,7 +17864,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>CP4 | Closet Outer → Aristech | Closet Outer | defined head</t>
+          <t>CP4 | Closet Outer → Aristech | Closet Outer | defined head | was S4-1</t>
         </is>
       </c>
     </row>
@@ -17919,7 +17889,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Head S4-2 G</t>
+          <t>Head 68L G</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -17934,7 +17904,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>CP4 | Closet Inner → Aristech | Closet Inner | defined head</t>
+          <t>CP4 | Closet Inner → Aristech | Closet Inner | defined head | was S4-2</t>
         </is>
       </c>
     </row>
@@ -17959,7 +17929,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Head S4-2 Y</t>
+          <t>Head 68L Y</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -17974,7 +17944,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>CP4 | Closet Inner → Aristech | Closet Inner | defined head</t>
+          <t>CP4 | Closet Inner → Aristech | Closet Inner | defined head | was S4-2</t>
         </is>
       </c>
     </row>
@@ -17999,7 +17969,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Head S4-2 R</t>
+          <t>Head 68L R</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -18014,7 +17984,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>CP4 | Closet Inner → Aristech | Closet Inner | defined head</t>
+          <t>CP4 | Closet Inner → Aristech | Closet Inner | defined head | was S4-2</t>
         </is>
       </c>
     </row>
@@ -18039,7 +18009,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Head S4-5 Y</t>
+          <t>Head 66RB Y</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -18054,7 +18024,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>CP4 | NIL B → Closet Inner | SW138 | mast SW138 (with S4-4)</t>
+          <t>CP4 | NIL B → Closet Inner | Switch 65 | mast Switch 65 (with 66RA) | was S4-5</t>
         </is>
       </c>
     </row>
@@ -18119,7 +18089,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Head S4-3 G</t>
+          <t>Head 64L G</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -18134,7 +18104,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>CP4 | Aristech → Closet Inner | SW127 | defined head</t>
+          <t>CP4 | Aristech → Closet Inner | Switch 63 | defined head | was S4-3</t>
         </is>
       </c>
     </row>
@@ -18159,7 +18129,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Head S4-3 Y</t>
+          <t>Head 64L Y</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -18174,7 +18144,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>CP4 | Aristech → Closet Inner | SW127 | defined head</t>
+          <t>CP4 | Aristech → Closet Inner | Switch 63 | defined head | was S4-3</t>
         </is>
       </c>
     </row>
@@ -18199,7 +18169,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Head S4-3 R</t>
+          <t>Head 64L R</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -18214,7 +18184,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>CP4 | Aristech → Closet Inner | SW127 | defined head</t>
+          <t>CP4 | Aristech → Closet Inner | Switch 63 | defined head | was S4-3</t>
         </is>
       </c>
     </row>
@@ -18239,7 +18209,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Head S4-4 G</t>
+          <t>Head 66RA G</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -18254,7 +18224,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>CP4 | Coke Plant → Closet Inner | SW138 | mast SW138 (with S4-5)</t>
+          <t>CP4 | Coke Plant → Closet Inner | Switch 65 | mast Switch 65 (with 66RB) | was S4-4</t>
         </is>
       </c>
     </row>
@@ -18279,7 +18249,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Head S4-4 Y</t>
+          <t>Head 66RA Y</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -18294,7 +18264,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>CP4 | Coke Plant → Closet Inner | SW138 | mast SW138 (with S4-5)</t>
+          <t>CP4 | Coke Plant → Closet Inner | Switch 65 | mast Switch 65 (with 66RB) | was S4-4</t>
         </is>
       </c>
     </row>
@@ -18319,7 +18289,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Head S4-4 R</t>
+          <t>Head 66RA R</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -18334,7 +18304,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>CP4 | Coke Plant → Closet Inner | SW138 | mast SW138 (with S4-5)</t>
+          <t>CP4 | Coke Plant → Closet Inner | Switch 65 | mast Switch 65 (with 66RB) | was S4-4</t>
         </is>
       </c>
     </row>
@@ -18359,7 +18329,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Head S4-5 G</t>
+          <t>Head 66RB G</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -18374,7 +18344,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>CP4 | NIL B → Closet Inner | SW138 | mast SW138 (with S4-4)</t>
+          <t>CP4 | NIL B → Closet Inner | Switch 65 | mast Switch 65 (with 66RA) | was S4-5</t>
         </is>
       </c>
     </row>
@@ -18399,7 +18369,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Head S4-5 R</t>
+          <t>Head 66RB R</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -18414,7 +18384,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>CP4 | NIL B → Closet Inner | SW138 | mast SW138 (with S4-4)</t>
+          <t>CP4 | NIL B → Closet Inner | Switch 65 | mast Switch 65 (with 66RA) | was S4-5</t>
         </is>
       </c>
     </row>
@@ -18439,7 +18409,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>DJE N</t>
+          <t>Switch 69 N</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -18474,7 +18444,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>DJE R</t>
+          <t>Switch 69 R</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -18509,7 +18479,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>DJW N</t>
+          <t>Switch 71 N</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -18544,7 +18514,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>DJW R</t>
+          <t>Switch 71 R</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -18719,7 +18689,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Head S5-1 G</t>
+          <t>Head 70L G</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -18734,7 +18704,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>CP5 | OutsideOuter → ClosetOuter | OutsideOuter | defined head</t>
+          <t>CP5 | OutsideOuter → ClosetOuter | OutsideOuter | defined head | was S5-1</t>
         </is>
       </c>
     </row>
@@ -18759,7 +18729,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Head S5-1 Y</t>
+          <t>Head 70L Y</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -18774,7 +18744,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>CP5 | OutsideOuter → ClosetOuter | OutsideOuter | defined head</t>
+          <t>CP5 | OutsideOuter → ClosetOuter | OutsideOuter | defined head | was S5-1</t>
         </is>
       </c>
     </row>
@@ -18799,7 +18769,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Head S5-1 R</t>
+          <t>Head 70L R</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -18814,7 +18784,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>CP5 | OutsideOuter → ClosetOuter | OutsideOuter | defined head</t>
+          <t>CP5 | OutsideOuter → ClosetOuter | OutsideOuter | defined head | was S5-1</t>
         </is>
       </c>
     </row>
@@ -18839,7 +18809,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Head S5-2 G</t>
+          <t>Head 72L G</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -18854,7 +18824,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>CP5 | ClosetOuter → OutsideOuter | ClosetOuter | defined head</t>
+          <t>CP5 | ClosetOuter → OutsideOuter | ClosetOuter | defined head | was S5-2</t>
         </is>
       </c>
     </row>
@@ -18879,7 +18849,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Head S5-2 Y</t>
+          <t>Head 72L Y</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -18894,7 +18864,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>CP5 | ClosetOuter → OutsideOuter | ClosetOuter | defined head</t>
+          <t>CP5 | ClosetOuter → OutsideOuter | ClosetOuter | defined head | was S5-2</t>
         </is>
       </c>
     </row>
@@ -18919,7 +18889,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Head S5-2 R</t>
+          <t>Head 72L R</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -18934,7 +18904,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>CP5 | ClosetOuter → OutsideOuter | ClosetOuter | defined head</t>
+          <t>CP5 | ClosetOuter → OutsideOuter | ClosetOuter | defined head | was S5-2</t>
         </is>
       </c>
     </row>
@@ -18959,7 +18929,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Head S5-5 Y</t>
+          <t>Head 70RA Y</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
@@ -18974,7 +18944,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>CP5 | Bridgeville → ClosetInner | Bridgeville | defined head</t>
+          <t>CP5 | Bridgeville → ClosetInner | Bridgeville | defined head | was S5-5</t>
         </is>
       </c>
     </row>
@@ -19039,7 +19009,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Head S5-3 G</t>
+          <t>Head 74L G</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -19054,7 +19024,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>CP5 | OutsideInner → ClosetInner | OutsideInner | defined head</t>
+          <t>CP5 | OutsideInner → ClosetInner | OutsideInner | defined head | was S5-3</t>
         </is>
       </c>
     </row>
@@ -19079,7 +19049,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Head S5-3 Y</t>
+          <t>Head 74L Y</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -19094,7 +19064,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>CP5 | OutsideInner → ClosetInner | OutsideInner | defined head</t>
+          <t>CP5 | OutsideInner → ClosetInner | OutsideInner | defined head | was S5-3</t>
         </is>
       </c>
     </row>
@@ -19119,7 +19089,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Head S5-3 R</t>
+          <t>Head 74L R</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -19134,7 +19104,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>CP5 | OutsideInner → ClosetInner | OutsideInner | defined head</t>
+          <t>CP5 | OutsideInner → ClosetInner | OutsideInner | defined head | was S5-3</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19129,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Head S5-4 G</t>
+          <t>Head 74RA G</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
@@ -19174,7 +19144,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>CP5 | ClosetInner → Bridgeville | ClosetInner | defined head</t>
+          <t>CP5 | ClosetInner → Bridgeville | ClosetInner | defined head | was S5-4</t>
         </is>
       </c>
     </row>
@@ -19199,7 +19169,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Head S5-4 Y</t>
+          <t>Head 74RA Y</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
@@ -19214,7 +19184,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>CP5 | ClosetInner → Bridgeville | ClosetInner | defined head</t>
+          <t>CP5 | ClosetInner → Bridgeville | ClosetInner | defined head | was S5-4</t>
         </is>
       </c>
     </row>
@@ -19239,7 +19209,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Head S5-4 R</t>
+          <t>Head 74RA R</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
@@ -19254,7 +19224,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>CP5 | ClosetInner → Bridgeville | ClosetInner | defined head</t>
+          <t>CP5 | ClosetInner → Bridgeville | ClosetInner | defined head | was S5-4</t>
         </is>
       </c>
     </row>
@@ -19279,7 +19249,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Head S5-5 G</t>
+          <t>Head 70RA G</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -19294,7 +19264,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>CP5 | Bridgeville → ClosetInner | Bridgeville | defined head</t>
+          <t>CP5 | Bridgeville → ClosetInner | Bridgeville | defined head | was S5-5</t>
         </is>
       </c>
     </row>
@@ -19319,7 +19289,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Head S5-5 R</t>
+          <t>Head 70RA R</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
@@ -19334,7 +19304,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>CP5 | Bridgeville → ClosetInner | Bridgeville | defined head</t>
+          <t>CP5 | Bridgeville → ClosetInner | Bridgeville | defined head | was S5-5</t>
         </is>
       </c>
     </row>
@@ -19359,7 +19329,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>SW124 N</t>
+          <t>Switch 73 N</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
@@ -19399,7 +19369,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>SW124 R</t>
+          <t>Switch 73 R</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
@@ -19589,7 +19559,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Head S5-6 G</t>
+          <t>Head 70RB G</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
@@ -19604,7 +19574,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>CP5 | HelixOuterB → Bridgeville | HelixOuterB | mast DJE reverse</t>
+          <t>CP5 | HelixOuterB → Bridgeville | HelixOuterB | mast Switch 69 reverse | was S5-6</t>
         </is>
       </c>
     </row>
@@ -19629,7 +19599,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Head S5-6 Y</t>
+          <t>Head 70RB Y</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
@@ -19644,7 +19614,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>CP5 | HelixOuterB → Bridgeville | HelixOuterB | mast DJE reverse</t>
+          <t>CP5 | HelixOuterB → Bridgeville | HelixOuterB | mast Switch 69 reverse | was S5-6</t>
         </is>
       </c>
     </row>
@@ -19669,7 +19639,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Head S5-6 R</t>
+          <t>Head 70RB R</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
@@ -19684,7 +19654,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>CP5 | HelixOuterB → Bridgeville | HelixOuterB | mast DJE reverse</t>
+          <t>CP5 | HelixOuterB → Bridgeville | HelixOuterB | mast Switch 69 reverse | was S5-6</t>
         </is>
       </c>
     </row>
@@ -19709,7 +19679,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Head S5-7 G</t>
+          <t>Head 74RB G</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
@@ -19724,7 +19694,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>CP5 | HelixInnerB → Bridgeville | HelixInnerB | mast SW124 reverse</t>
+          <t>CP5 | HelixInnerB → Bridgeville | HelixInnerB | mast Switch 73 reverse | was S5-7</t>
         </is>
       </c>
     </row>
@@ -19749,7 +19719,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Head S5-7 R</t>
+          <t>Head 74RB R</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
@@ -19764,7 +19734,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>CP5 | HelixInnerB → Bridgeville | HelixInnerB | mast SW124 reverse</t>
+          <t>CP5 | HelixInnerB → Bridgeville | HelixInnerB | mast Switch 73 reverse | was S5-7</t>
         </is>
       </c>
     </row>
@@ -19789,7 +19759,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Head S5-7 Y</t>
+          <t>Head 74RB Y</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
@@ -19804,7 +19774,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>CP5 | HelixInnerB → Bridgeville | HelixInnerB | mast SW124 reverse</t>
+          <t>CP5 | HelixInnerB → Bridgeville | HelixInnerB | mast Switch 73 reverse | was S5-7</t>
         </is>
       </c>
     </row>
@@ -19879,7 +19849,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>CBX N</t>
+          <t>Switch 75 N</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
@@ -19914,7 +19884,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>CBX R</t>
+          <t>Switch 75 R</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
@@ -19949,7 +19919,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>SW143 N</t>
+          <t>Switch 77 N</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
@@ -19989,7 +19959,7 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>SW143 R</t>
+          <t>Switch 77 R</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
@@ -20159,7 +20129,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Head S6-6 G</t>
+          <t>Head 78R G</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
@@ -20174,7 +20144,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>CP6 | CBOuter → CBStation | CBOuter | defined head</t>
+          <t>CP6 | CBOuter → CBStation | CBOuter | defined head | was S6-6</t>
         </is>
       </c>
     </row>
@@ -20199,7 +20169,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Head S6-6 Y</t>
+          <t>Head 78R Y</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
@@ -20214,7 +20184,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>CP6 | CBOuter → CBStation | CBOuter | defined head</t>
+          <t>CP6 | CBOuter → CBStation | CBOuter | defined head | was S6-6</t>
         </is>
       </c>
     </row>
@@ -20239,7 +20209,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Head S6-6 R</t>
+          <t>Head 78R R</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
@@ -20254,7 +20224,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>CP6 | CBOuter → CBStation | CBOuter | defined head</t>
+          <t>CP6 | CBOuter → CBStation | CBOuter | defined head | was S6-6</t>
         </is>
       </c>
     </row>
@@ -20279,7 +20249,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Head S6-8 G</t>
+          <t>Head 88R G</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
@@ -20294,7 +20264,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>CP6 | CBSiding → CBInner | CBSiding | defined head</t>
+          <t>CP6 | CBSiding → CBInner | CBSiding | defined head | was S6-8</t>
         </is>
       </c>
     </row>
@@ -20319,7 +20289,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Head S6-8 Y</t>
+          <t>Head 88R Y</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
@@ -20334,7 +20304,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>CP6 | CBSiding → CBInner | CBSiding | defined head</t>
+          <t>CP6 | CBSiding → CBInner | CBSiding | defined head | was S6-8</t>
         </is>
       </c>
     </row>
@@ -20359,7 +20329,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Head S6-8 R</t>
+          <t>Head 88R R</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
@@ -20374,7 +20344,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>CP6 | CBSiding → CBInner | CBSiding | defined head</t>
+          <t>CP6 | CBSiding → CBInner | CBSiding | defined head | was S6-8</t>
         </is>
       </c>
     </row>
@@ -20399,7 +20369,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Head S6-12 Y</t>
+          <t>Head 84RB Y</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
@@ -20414,7 +20384,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW147 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 85 | defined head | was S6-12</t>
         </is>
       </c>
     </row>
@@ -20479,7 +20449,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Head S6-15 G</t>
+          <t>Head 92L G</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
@@ -20494,7 +20464,7 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW150 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 91 | defined head | was S6-15</t>
         </is>
       </c>
     </row>
@@ -20519,7 +20489,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Head S6-15 R</t>
+          <t>Head 92L R</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
@@ -20534,7 +20504,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW150 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 91 | defined head | was S6-15</t>
         </is>
       </c>
     </row>
@@ -20559,7 +20529,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Head S6-15 Y</t>
+          <t>Head 92L Y</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
@@ -20574,7 +20544,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW150 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 91 | defined head | was S6-15</t>
         </is>
       </c>
     </row>
@@ -20599,7 +20569,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Head S6-14 G</t>
+          <t>Head 90L G</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
@@ -20614,7 +20584,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW149 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 89 | defined head | was S6-14</t>
         </is>
       </c>
     </row>
@@ -20639,7 +20609,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Head S6-14 R</t>
+          <t>Head 90L R</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
@@ -20654,7 +20624,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW149 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 89 | defined head | was S6-14</t>
         </is>
       </c>
     </row>
@@ -20679,7 +20649,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Head S6-14 Y</t>
+          <t>Head 90L Y</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
@@ -20694,7 +20664,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW149 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 89 | defined head | was S6-14</t>
         </is>
       </c>
     </row>
@@ -20719,7 +20689,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Head S6-12 G</t>
+          <t>Head 84RB G</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
@@ -20734,7 +20704,7 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW147 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 85 | defined head | was S6-12</t>
         </is>
       </c>
     </row>
@@ -20759,7 +20729,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Head S6-12 R</t>
+          <t>Head 84RB R</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
@@ -20774,7 +20744,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW147 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 85 | defined head | was S6-12</t>
         </is>
       </c>
     </row>
@@ -20799,7 +20769,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>SW144 N</t>
+          <t>Switch 79 N</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -20839,7 +20809,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>SW144 R</t>
+          <t>Switch 79 R</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
@@ -20879,7 +20849,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>SW145 N</t>
+          <t>Switch 81 N</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
@@ -20919,7 +20889,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>SW145 R</t>
+          <t>Switch 81 R</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
@@ -20959,7 +20929,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>SW146 N</t>
+          <t>Switch 83 N</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
@@ -20999,7 +20969,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>SW146 R</t>
+          <t>Switch 83 R</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
@@ -21039,7 +21009,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>SW147 N</t>
+          <t>Switch 85 N</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -21079,7 +21049,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>SW147 R</t>
+          <t>Switch 85 R</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -21119,7 +21089,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Head S6-2 G</t>
+          <t>Head 76R G</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -21134,7 +21104,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>CP6 | OutsideInnerA → CBInner | OutsideInnerA | defined head</t>
+          <t>CP6 | OutsideInnerA → CBInner | OutsideInnerA | defined head | was S6-2</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21129,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Head S6-2 Y</t>
+          <t>Head 76R Y</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -21174,7 +21144,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>CP6 | OutsideInnerA → CBInner | OutsideInnerA | defined head</t>
+          <t>CP6 | OutsideInnerA → CBInner | OutsideInnerA | defined head | was S6-2</t>
         </is>
       </c>
     </row>
@@ -21199,7 +21169,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Head S6-2 R</t>
+          <t>Head 76R R</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -21214,7 +21184,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>CP6 | OutsideInnerA → CBInner | OutsideInnerA | defined head</t>
+          <t>CP6 | OutsideInnerA → CBInner | OutsideInnerA | defined head | was S6-2</t>
         </is>
       </c>
     </row>
@@ -21239,7 +21209,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>Head S6-13 G</t>
+          <t>Head 86L G</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
@@ -21254,7 +21224,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW148 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 87 | defined head | was S6-13</t>
         </is>
       </c>
     </row>
@@ -21279,7 +21249,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Head S6-13 R</t>
+          <t>Head 86L R</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
@@ -21294,7 +21264,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW148 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 87 | defined head | was S6-13</t>
         </is>
       </c>
     </row>
@@ -21319,7 +21289,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Head S6-13 Y</t>
+          <t>Head 86L Y</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
@@ -21334,7 +21304,7 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW148 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 87 | defined head | was S6-13</t>
         </is>
       </c>
     </row>
@@ -21359,7 +21329,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>Head S6-11 Y</t>
+          <t>Head 84RA Y</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
@@ -21374,7 +21344,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW146 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 83 | defined head | was S6-11</t>
         </is>
       </c>
     </row>
@@ -21439,7 +21409,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Head S6-1 G</t>
+          <t>Head 76L G</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -21454,7 +21424,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>CP6 | OutsideOuterA → CBInner | OutsideOuterA | defined head</t>
+          <t>CP6 | OutsideOuterA → CBInner | OutsideOuterA | defined head | was S6-1</t>
         </is>
       </c>
     </row>
@@ -21479,7 +21449,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Head S6-1 Y</t>
+          <t>Head 76L Y</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -21494,7 +21464,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>CP6 | OutsideOuterA → CBInner | OutsideOuterA | defined head</t>
+          <t>CP6 | OutsideOuterA → CBInner | OutsideOuterA | defined head | was S6-1</t>
         </is>
       </c>
     </row>
@@ -21519,7 +21489,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Head S6-1 R</t>
+          <t>Head 76L R</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -21534,7 +21504,7 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>CP6 | OutsideOuterA → CBInner | OutsideOuterA | defined head</t>
+          <t>CP6 | OutsideOuterA → CBInner | OutsideOuterA | defined head | was S6-1</t>
         </is>
       </c>
     </row>
@@ -21559,7 +21529,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Head S6-5 G</t>
+          <t>Head 78RB G</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
@@ -21574,7 +21544,7 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>CP6 | CBSiding → OutsideInnerA | CBSiding | defined head</t>
+          <t>CP6 | CBSiding → OutsideInnerA | CBSiding | defined head | was S6-5</t>
         </is>
       </c>
     </row>
@@ -21599,7 +21569,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Head S6-5 Y</t>
+          <t>Head 78RB Y</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -21614,7 +21584,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>CP6 | CBSiding → OutsideInnerA | CBSiding | defined head</t>
+          <t>CP6 | CBSiding → OutsideInnerA | CBSiding | defined head | was S6-5</t>
         </is>
       </c>
     </row>
@@ -21639,7 +21609,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Head S6-5 R</t>
+          <t>Head 78RB R</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
@@ -21654,7 +21624,7 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>CP6 | CBSiding → OutsideInnerA | CBSiding | defined head</t>
+          <t>CP6 | CBSiding → OutsideInnerA | CBSiding | defined head | was S6-5</t>
         </is>
       </c>
     </row>
@@ -21679,7 +21649,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Head S6-11 G</t>
+          <t>Head 84RA G</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -21694,7 +21664,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW146 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 83 | defined head | was S6-11</t>
         </is>
       </c>
     </row>
@@ -21719,7 +21689,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Head S6-11 R</t>
+          <t>Head 84RA R</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
@@ -21734,7 +21704,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW146 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 83 | defined head | was S6-11</t>
         </is>
       </c>
     </row>
@@ -21759,7 +21729,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>SW148 N</t>
+          <t>Switch 87 N</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -21799,7 +21769,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>SW148 R</t>
+          <t>Switch 87 R</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -21839,7 +21809,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>SW149 N</t>
+          <t>Switch 89 N</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
@@ -21879,7 +21849,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>SW149 R</t>
+          <t>Switch 89 R</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
@@ -21919,7 +21889,7 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>SW150 N</t>
+          <t>Switch 91 N</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
@@ -21959,7 +21929,7 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>SW150 R</t>
+          <t>Switch 91 R</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
@@ -21999,7 +21969,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>Head S6-10 G</t>
+          <t>Head 82L G</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
@@ -22014,7 +21984,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW144 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 79 | defined head | was S6-10</t>
         </is>
       </c>
     </row>
@@ -22039,7 +22009,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>Head S6-10 R</t>
+          <t>Head 82L R</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
@@ -22054,7 +22024,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW144 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 79 | defined head | was S6-10</t>
         </is>
       </c>
     </row>
@@ -22079,7 +22049,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>Head S6-3 G</t>
+          <t>Head 78L G</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -22094,7 +22064,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>CP6 | CBStation → CBOuter | CBStation | defined head</t>
+          <t>CP6 | CBStation → CBOuter | CBStation | defined head | was S6-3</t>
         </is>
       </c>
     </row>
@@ -22119,7 +22089,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>Head S6-3 Y</t>
+          <t>Head 78L Y</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -22134,7 +22104,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>CP6 | CBStation → CBOuter | CBStation | defined head</t>
+          <t>CP6 | CBStation → CBOuter | CBStation | defined head | was S6-3</t>
         </is>
       </c>
     </row>
@@ -22159,7 +22129,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Head S6-3 R</t>
+          <t>Head 78L R</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -22174,7 +22144,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>CP6 | CBStation → CBOuter | CBStation | defined head</t>
+          <t>CP6 | CBStation → CBOuter | CBStation | defined head | was S6-3</t>
         </is>
       </c>
     </row>
@@ -22199,7 +22169,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>Head S6-9 G</t>
+          <t>Head 88RA G</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -22214,7 +22184,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>CP6 | CB Outer → CB Station | CB Outer | defined head</t>
+          <t>CP6 | CB Outer → CB Station | CB Outer | defined head | was S6-9</t>
         </is>
       </c>
     </row>
@@ -22239,7 +22209,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Head S6-9 Y</t>
+          <t>Head 88RA Y</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -22254,7 +22224,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>CP6 | CB Outer → CB Station | CB Outer | defined head</t>
+          <t>CP6 | CB Outer → CB Station | CB Outer | defined head | was S6-9</t>
         </is>
       </c>
     </row>
@@ -22279,7 +22249,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Head S6-9 R</t>
+          <t>Head 88RA R</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
@@ -22294,7 +22264,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>CP6 | CB Outer → CB Station | CB Outer | defined head</t>
+          <t>CP6 | CB Outer → CB Station | CB Outer | defined head | was S6-9</t>
         </is>
       </c>
     </row>
@@ -22319,7 +22289,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Head S6-10 Y</t>
+          <t>Head 82L Y</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
@@ -22334,7 +22304,7 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>CP6 | ? → OutsideOuterA | SW144 | defined head</t>
+          <t>CP6 | ? → OutsideOuterA | Switch 79 | defined head | was S6-10</t>
         </is>
       </c>
     </row>
@@ -22399,7 +22369,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Head S6-4 G</t>
+          <t>Head 78RA G</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -22414,7 +22384,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>CP6 | CBStation → OutsideInnerA | CBStation | defined head</t>
+          <t>CP6 | CBStation → OutsideInnerA | CBStation | defined head | was S6-4</t>
         </is>
       </c>
     </row>
@@ -22439,7 +22409,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Head S6-4 Y</t>
+          <t>Head 78RA Y</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -22454,7 +22424,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>CP6 | CBStation → OutsideInnerA | CBStation | defined head</t>
+          <t>CP6 | CBStation → OutsideInnerA | CBStation | defined head | was S6-4</t>
         </is>
       </c>
     </row>
@@ -22479,7 +22449,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Head S6-4 R</t>
+          <t>Head 78RA R</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -22494,7 +22464,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>CP6 | CBStation → OutsideInnerA | CBStation | defined head</t>
+          <t>CP6 | CBStation → OutsideInnerA | CBStation | defined head | was S6-4</t>
         </is>
       </c>
     </row>
@@ -22519,7 +22489,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Head S6-7 G</t>
+          <t>Head 88L G</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
@@ -22534,7 +22504,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>CP6 | CBInner → CBSiding | CBInner | defined head</t>
+          <t>CP6 | CBInner → CBSiding | CBInner | defined head | was S6-7</t>
         </is>
       </c>
     </row>
@@ -22559,7 +22529,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Head S6-7 Y</t>
+          <t>Head 88L Y</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
@@ -22574,7 +22544,7 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>CP6 | CBInner → CBSiding | CBInner | defined head</t>
+          <t>CP6 | CBInner → CBSiding | CBInner | defined head | was S6-7</t>
         </is>
       </c>
     </row>
@@ -22599,7 +22569,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Head S6-7 R</t>
+          <t>Head 88L R</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -22614,7 +22584,7 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>CP6 | CBInner → CBSiding | CBInner | defined head</t>
+          <t>CP6 | CBInner → CBSiding | CBInner | defined head | was S6-7</t>
         </is>
       </c>
     </row>
@@ -26465,7 +26435,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>NIX N FB</t>
+          <t>Switch 61 N FB</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -26495,7 +26465,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>NIX R FB</t>
+          <t>Switch 61 R FB</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -26525,7 +26495,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>SW129 N FB</t>
+          <t>Switch 67 N FB</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -26560,7 +26530,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>SW129 R FB</t>
+          <t>Switch 67 R FB</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -26595,7 +26565,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>SW127 N FB</t>
+          <t>Switch 63 N FB</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -26630,7 +26600,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>SW127 R FB</t>
+          <t>Switch 63 R FB</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -26665,7 +26635,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>SW138 N FB</t>
+          <t>Switch 65 N FB</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -26700,7 +26670,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>SW138 R FB</t>
+          <t>Switch 65 R FB</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -26735,7 +26705,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>NIX BTN</t>
+          <t>Switch 61 BTN</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -26765,7 +26735,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>SW129 BTN</t>
+          <t>Switch 67 BTN</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -26800,7 +26770,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>SW127 BTN</t>
+          <t>Switch 63 BTN</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -26835,7 +26805,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>SW138 BTN</t>
+          <t>Switch 65 BTN</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -26950,7 +26920,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>DJE N FB</t>
+          <t>Switch 69 N FB</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -26980,7 +26950,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>DJE R FB</t>
+          <t>Switch 69 R FB</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -27010,7 +26980,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>DJW N FB</t>
+          <t>Switch 71 N FB</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -27040,7 +27010,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>DJW R FB</t>
+          <t>Switch 71 R FB</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -27070,7 +27040,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>SW124 N FB</t>
+          <t>Switch 73 N FB</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -27105,7 +27075,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>SW124 R FB</t>
+          <t>Switch 73 R FB</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -27180,7 +27150,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>DJE BTN</t>
+          <t>Switch 69 BTN</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -27210,7 +27180,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>DJW BTN</t>
+          <t>Switch 71 BTN</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -27240,7 +27210,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>SW124 BTN</t>
+          <t>Switch 73 BTN</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -27375,7 +27345,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>CBX N FB</t>
+          <t>Switch 75 N FB</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -27405,7 +27375,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>CBX R FB</t>
+          <t>Switch 75 R FB</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -27435,7 +27405,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>SW143 N FB</t>
+          <t>Switch 77 N FB</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -27470,7 +27440,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>SW143 R FB</t>
+          <t>Switch 77 R FB</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -27545,7 +27515,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>CBX BTN</t>
+          <t>Switch 75 BTN</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -27575,7 +27545,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>SW143 BTN</t>
+          <t>Switch 77 BTN</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -27610,7 +27580,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>SW144 N FB</t>
+          <t>Switch 79 N FB</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -27645,7 +27615,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>SW144 R FB</t>
+          <t>Switch 79 R FB</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -27680,7 +27650,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>SW145 N FB</t>
+          <t>Switch 81 N FB</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -27715,7 +27685,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>SW145 R FB</t>
+          <t>Switch 81 R FB</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -27750,7 +27720,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>SW146 N FB</t>
+          <t>Switch 83 N FB</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -27785,7 +27755,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>SW146 R FB</t>
+          <t>Switch 83 R FB</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -27820,7 +27790,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>SW147 N FB</t>
+          <t>Switch 85 N FB</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -27855,7 +27825,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>SW147 R FB</t>
+          <t>Switch 85 R FB</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -27890,7 +27860,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>SW144 BTN</t>
+          <t>Switch 79 BTN</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -27925,7 +27895,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>SW145 BTN</t>
+          <t>Switch 81 BTN</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -27960,7 +27930,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>SW146 BTN</t>
+          <t>Switch 83 BTN</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -27995,7 +27965,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>SW147 BTN</t>
+          <t>Switch 85 BTN</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -28110,7 +28080,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>SW148 N FB</t>
+          <t>Switch 87 N FB</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -28145,7 +28115,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>SW148 R FB</t>
+          <t>Switch 87 R FB</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -28180,7 +28150,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>SW149 N FB</t>
+          <t>Switch 89 N FB</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -28215,7 +28185,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>SW149 R FB</t>
+          <t>Switch 89 R FB</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -28250,7 +28220,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>SW150 N FB</t>
+          <t>Switch 91 N FB</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -28285,7 +28255,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>SW150 R FB</t>
+          <t>Switch 91 R FB</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -28360,7 +28330,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>SW148 BTN</t>
+          <t>Switch 87 BTN</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -28395,7 +28365,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>SW149 BTN</t>
+          <t>Switch 89 BTN</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -28430,7 +28400,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>SW150 BTN</t>
+          <t>Switch 91 BTN</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -29341,7 +29311,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SW127</t>
+          <t>Switch 63</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -29356,7 +29326,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>SW127</t>
+          <t>Switch 63</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -29376,7 +29346,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>S4-3</t>
+          <t>64L</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -29396,7 +29366,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>S4-1</t>
+          <t>64R</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -29418,7 +29388,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SW129</t>
+          <t>Switch 67</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -29433,7 +29403,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SW129</t>
+          <t>Switch 67</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -29453,7 +29423,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>S4-2</t>
+          <t>68L</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -29475,7 +29445,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SW138</t>
+          <t>Switch 65</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -29490,7 +29460,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SW138</t>
+          <t>Switch 65</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -29510,7 +29480,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>S4-4</t>
+          <t>66RA</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -29530,7 +29500,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>S4-5</t>
+          <t>66RB</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -29823,7 +29793,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NIX</t>
+          <t>Switch 61</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -29838,7 +29808,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SW125, SW126, SW139, SW140</t>
+          <t>Switch 61a, Switch 61b, Switch 61c, Switch 61d</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -29858,7 +29828,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>S4-6</t>
+          <t>62L</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -29878,7 +29848,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>S4-5</t>
+          <t>66RB</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -29898,7 +29868,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>S4-4</t>
+          <t>66RA</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -30127,46 +30097,6 @@
           <t>C12-IN1-6</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>S2-8</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>C12-OU3-8</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>C12-OU2-7</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>C12-OU3-7</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>S2-5</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>C2-OU2-3</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>C2-OU2-2</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>C2-OU2-1</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -30276,26 +30206,6 @@
           <t>C12-IN1-2</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>S2-6</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>C2-OU3-2</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>C2-OU2-7</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>C2-OU3-1</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -30333,31 +30243,11 @@
           <t>C12-IN1-4</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>S2-7</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>C2-OU3-4</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>C2-OU3-5</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>C2-OU3-3</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SW124</t>
+          <t>Switch 73</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -30372,7 +30262,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SW124</t>
+          <t>Switch 73</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -30392,7 +30282,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>S5-3</t>
+          <t>74L</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -30412,7 +30302,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>S5-4</t>
+          <t>74RA</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -30432,7 +30322,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>S5-7</t>
+          <t>74RB</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -30454,7 +30344,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DJE</t>
+          <t>Switch 69</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -30469,7 +30359,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>SW121, SW123</t>
+          <t>Switch 69a, Switch 69b</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -30489,7 +30379,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>S5-1</t>
+          <t>70L</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -30509,7 +30399,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>S5-5</t>
+          <t>70RA</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -30529,7 +30419,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>S5-6</t>
+          <t>70RB</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -30551,7 +30441,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DJW</t>
+          <t>Switch 71</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -30566,7 +30456,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>SW120, SW122</t>
+          <t>Switch 71a, Switch 71b</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -30586,7 +30476,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>S5-2</t>
+          <t>72L</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -30606,7 +30496,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>S5-4</t>
+          <t>74RA</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -30839,7 +30729,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SW148</t>
+          <t>Switch 87</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -30854,7 +30744,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>SW148</t>
+          <t>Switch 87</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -30874,7 +30764,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>S6-1</t>
+          <t>76L</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -30894,7 +30784,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>S6-5</t>
+          <t>78RB</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -30916,7 +30806,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SW149</t>
+          <t>Switch 89</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -30931,7 +30821,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>SW149</t>
+          <t>Switch 89</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -30951,7 +30841,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>S6-14</t>
+          <t>90L</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -30973,7 +30863,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SW150</t>
+          <t>Switch 91</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -30988,7 +30878,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>SW150</t>
+          <t>Switch 91</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -31008,7 +30898,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>S6-15</t>
+          <t>92L</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -31178,7 +31068,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CBX</t>
+          <t>Switch 75</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -31193,7 +31083,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>SW141, SW142</t>
+          <t>Switch 75a, Switch 75b</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -31213,7 +31103,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>S6-1</t>
+          <t>76L</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -31233,7 +31123,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>S6-2</t>
+          <t>76R</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -31255,7 +31145,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SW143</t>
+          <t>Switch 77</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -31270,7 +31160,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SW143</t>
+          <t>Switch 77</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -31290,7 +31180,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>S6-4</t>
+          <t>78RA</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -31310,7 +31200,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>S6-5</t>
+          <t>78RB</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -31332,7 +31222,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SW144</t>
+          <t>Switch 79</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -31347,7 +31237,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>SW144</t>
+          <t>Switch 79</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -31367,7 +31257,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>S6-1</t>
+          <t>76L</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -31387,7 +31277,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>S6-4</t>
+          <t>78RA</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -31409,7 +31299,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SW145</t>
+          <t>Switch 81</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -31424,7 +31314,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>SW145</t>
+          <t>Switch 81</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -31444,7 +31334,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>S6-10</t>
+          <t>82L</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -31466,7 +31356,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SW146</t>
+          <t>Switch 83</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -31481,7 +31371,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>SW146</t>
+          <t>Switch 83</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -31501,7 +31391,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>S6-11</t>
+          <t>84RA</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -31521,7 +31411,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>S6-12</t>
+          <t>84RB</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -31543,7 +31433,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SW147</t>
+          <t>Switch 85</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -31558,7 +31448,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>SW147</t>
+          <t>Switch 85</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -33723,7 +33613,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Helix Inner A, SW124</t>
+          <t>Helix Inner A, Switch 73</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -33763,7 +33653,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Helix Outer A, SW121</t>
+          <t>Helix Outer A, Switch 69a</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -33803,7 +33693,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>SW138, NIL B</t>
+          <t>Switch 65, NIL B</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -33843,7 +33733,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>NIL B, SW129</t>
+          <t>NIL B, Switch 67</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -33878,7 +33768,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SW129</t>
+          <t>Switch 67</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -33923,7 +33813,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>SW127, SW129</t>
+          <t>Switch 63, Switch 67</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -33958,12 +33848,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SW127</t>
+          <t>Switch 63</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>SW128, Outer Leg, SW126</t>
+          <t>SW128, Outer Leg, Switch 61b</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -33998,12 +33888,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SW138</t>
+          <t>Switch 65</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>NIL A, SW137, SW139</t>
+          <t>NIL A, SW137, Switch 61c</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -34038,12 +33928,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SW139,140</t>
+          <t>Switch 61c,140</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>SW138, Closet Outer</t>
+          <t>Switch 65, Closet Outer</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -34078,12 +33968,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SW125,126</t>
+          <t>Switch 61a,126</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>SW127, SW123</t>
+          <t>Switch 63, Switch 69b</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -34123,7 +34013,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>SW140, SW124</t>
+          <t>Switch 61d, Switch 73</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -34163,7 +34053,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>SW125, Outside Outer B</t>
+          <t>Switch 61a, Outside Outer B</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -34198,12 +34088,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>SW124</t>
+          <t>Switch 73</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Closet Inner, SW123, Helix Inner B</t>
+          <t>Closet Inner, Switch 69b, Helix Inner B</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -34238,12 +34128,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>SW122,123</t>
+          <t>Switch 71b,123</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>SW124, Outside Inner B, SW120, SW121</t>
+          <t>Switch 73, Outside Inner B, Switch 71a, Switch 69a</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -34278,12 +34168,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>SW120</t>
+          <t>Switch 71a</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Bridgeville, SW121, SW122</t>
+          <t>Bridgeville, Switch 69a, Switch 71b</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -34318,12 +34208,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>SW121</t>
+          <t>Switch 69a</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Helix Outer B, SW120, SW123</t>
+          <t>Helix Outer B, Switch 71a, Switch 69b</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -34363,7 +34253,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Outside Outer B, SW141</t>
+          <t>Outside Outer B, Switch 75a</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -34403,7 +34293,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outside Inner B, SW142, </t>
+          <t xml:space="preserve">Outside Inner B, Switch 75b, </t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -34443,7 +34333,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Outside Inner A, SW122</t>
+          <t>Outside Inner A, Switch 71b</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -34483,7 +34373,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Outside Outer A, SW141</t>
+          <t>Outside Outer A, Switch 75a</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -34658,7 +34548,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>SW141</t>
+          <t>Switch 75a</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -34693,7 +34583,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>SW142</t>
+          <t>Switch 75b</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -34728,7 +34618,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>SW143</t>
+          <t>Switch 77</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -34763,7 +34653,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>SW144</t>
+          <t>Switch 79</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -34798,7 +34688,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>SW145</t>
+          <t>Switch 81</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -34833,7 +34723,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>SW146</t>
+          <t>Switch 83</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -34868,7 +34758,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>SW147</t>
+          <t>Switch 85</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -35008,7 +34898,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>SW148</t>
+          <t>Switch 87</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -35043,7 +34933,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>SW149</t>
+          <t>Switch 89</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -35078,7 +34968,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>SW150</t>
+          <t>Switch 91</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">

</xml_diff>

<commit_message>
Strip leftover S2-6/S2-7 names from C2 spare-pin notes so they no longer appear in the inventory.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
+++ b/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
@@ -14069,7 +14069,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>spare (CP2 leftover RGB removed; was S2-6 Y)</t>
+          <t>spare</t>
         </is>
       </c>
     </row>
@@ -14134,7 +14134,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>spare (CP2 leftover RGB removed; was S2-6 G)</t>
+          <t>spare</t>
         </is>
       </c>
     </row>
@@ -14164,7 +14164,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>spare (CP2 leftover RGB removed; was S2-6 R)</t>
+          <t>spare</t>
         </is>
       </c>
     </row>
@@ -14194,7 +14194,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>spare (CP2 leftover RGB removed; was S2-7 G)</t>
+          <t>spare</t>
         </is>
       </c>
     </row>
@@ -14224,7 +14224,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>spare (CP2 leftover RGB removed; was S2-7 R)</t>
+          <t>spare</t>
         </is>
       </c>
     </row>
@@ -14254,7 +14254,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>spare (CP2 leftover RGB removed; was S2-7 Y)</t>
+          <t>spare</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document Digicon Stop/Approach/Clear as R-Y-G on increasing LCOS ports.
Field wiring is Stop then Approach then Clear; the old docs had Stop and Clear reversed. Also record Signal Manager Main/Diverged and OR Stop/Approach per disc.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
+++ b/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Head 6LB T G</t>
+          <t>Head 6LB T R</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S3-6 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was S3-6 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp Y; was S3-6 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp Y; was S3-6 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Head 6LB T R</t>
+          <t>Head 6LB T G</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was S3-6 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S3-6 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Head 6LB B G</t>
+          <t>Head 6LB B R</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 6LB T on OU2</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 6LB T on OU2</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Head 6LB B R</t>
+          <t>Head 6LB B G</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 6LB T on OU2</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 6LB T on OU2</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Head 6LA G</t>
+          <t>Head 6LA R</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G on Plane OU2; Y/R on 2L OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was R on Plane OU2; Y/G on 2L OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was G on Plane OU2; Y/R on 2L OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was R on Plane OU2; Y/G on 2L OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Head 6LA R</t>
+          <t>Head 6LA G</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was G on Plane OU2; Y/R on 2L OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was R on Plane OU2; Y/G on 2L OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Head 2L T G</t>
+          <t>Head 2L T R</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was S3-8 G/Y/R</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was S3-8 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp Y; was S3-8 G/Y/R</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp Y; was S3-8 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Head 2L T R</t>
+          <t>Head 2L T G</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was S3-8 G/Y/R</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was S3-8 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Head 2L B G</t>
+          <t>Head 2L B R</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was with 2L T on OU3</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp R; was with 2L T on OU3</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Head 2L B R</t>
+          <t>Head 2L B G</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1619,7 +1619,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp R; was with 2L T on OU3</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was with 2L T on OU3</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Head 4RA G</t>
+          <t>Head 4RA R</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was Brick west OU4 with 4RB</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was Brick west OU4 with 4RB</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Head 4RA R</t>
+          <t>Head 4RA G</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was Brick west OU4 with 4RB</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was Brick west OU4 with 4RB</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Head 4RB G</t>
+          <t>Head 4RB R</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp G; was Brick west OU4 with 4RA</t>
+          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp R; was Brick west OU4 with 4RA</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Head 4RB R</t>
+          <t>Head 4RB G</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp R; was Brick west OU4 with 4RA</t>
+          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp G; was Brick west OU4 with 4RA</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Head 8RA T G</t>
+          <t>Head 8RA T R</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S3-10 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was S3-10 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp Y; was S3-10 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp Y; was S3-10 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Head 8RA T R</t>
+          <t>Head 8RA T G</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was S3-10 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S3-10 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Head 8RA B G</t>
+          <t>Head 8RA B R</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 8RA T on OU1</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 8RA T on OU1</t>
         </is>
       </c>
     </row>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Head 8RA B R</t>
+          <t>Head 8RA B G</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 8RA T on OU1</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 8RA T on OU1</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2535,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Head 8RB T G</t>
+          <t>Head 8RB T R</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2555,7 +2555,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was S3-12; sequential G/Y/R</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was S3-12; sequential R/Y/G</t>
         </is>
       </c>
     </row>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp Y; was S3-12; sequential G/Y/R</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp Y; was S3-12; sequential R/Y/G</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Head 8RB T R</t>
+          <t>Head 8RB T G</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was S3-12; sequential G/Y/R</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was S3-12; sequential R/Y/G</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Head 8RB B G</t>
+          <t>Head 8RB B R</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was with 8RB T on OU4</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was with 8RB T on OU4</t>
         </is>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Head 8RB B R</t>
+          <t>Head 8RB B G</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was with 8RB T on OU4</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was with 8RB T on OU4</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Head 8LA T G</t>
+          <t>Head 8LA T R</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp G; was S3-5 G/Y/R</t>
+          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp R; was S3-5 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -3069,7 +3069,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp Y; was S3-5 G/Y/R</t>
+          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp Y; was S3-5 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Head 8LA T R</t>
+          <t>Head 8LA T G</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3141,7 +3141,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp R; was S3-5 G/Y/R</t>
+          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp G; was S3-5 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Head 8LA B G</t>
+          <t>Head 8LA B R</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was with 8LA T on OU2</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was with 8LA T on OU2</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Head 8LA B R</t>
+          <t>Head 8LA B G</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3357,7 +3357,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was with 8LA T on OU2</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was with 8LA T on OU2</t>
         </is>
       </c>
     </row>
@@ -3399,7 +3399,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Head 8LB G</t>
+          <t>Head 8LB R</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G/Y with 8LA; R spills to 8RB OU4</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was R/Y with 8LA; G spills to 8RB OU4</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was G/Y with 8LA; R spills to 8RB OU4</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was R/Y with 8LA; G spills to 8RB OU4</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3543,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Head 8LB R</t>
+          <t>Head 8LB G</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was G/Y with 8LA; R spills to 8RB OU4</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was R/Y with 8LA; G spills to 8RB OU4</t>
         </is>
       </c>
     </row>
@@ -3615,7 +3615,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Head 24RA T G</t>
+          <t>Head 24RA T R</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -3645,7 +3645,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was C2-OU1 5V</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was C2-OU1 5V</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Head 24RA T R</t>
+          <t>Head 24RA T G</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was C2-OU1 5V</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was C2-OU1 5V</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Head 24RA B G</t>
+          <t>Head 24RA B R</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -3861,7 +3861,7 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was with 24RA T on OU1</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was with 24RA T on OU1</t>
         </is>
       </c>
     </row>
@@ -3975,7 +3975,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Head 24RA B R</t>
+          <t>Head 24RA B G</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -4005,7 +4005,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was with 24RA T on OU1</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was with 24RA T on OU1</t>
         </is>
       </c>
     </row>
@@ -4047,7 +4047,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Head 24RB G</t>
+          <t>Head 24RB R</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was whole dwarf on leftover OU3 (OU1-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was whole dwarf on leftover OU3 (OU1-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Head 24RB R</t>
+          <t>Head 24RB G</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -4221,7 +4221,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was whole dwarf on leftover OU3 (OU1-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was whole dwarf on leftover OU3 (OU1-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4263,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Head 24L T G</t>
+          <t>Head 24L T R</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -4293,7 +4293,7 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 24RA cluster</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 24RA cluster</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Head 24L T R</t>
+          <t>Head 24L T G</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -4437,7 +4437,7 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 24RA cluster</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 24RA cluster</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Head 24L B G</t>
+          <t>Head 24L B R</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was with 24L T on OU2</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp R; was with 24L T on OU2</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Head 24L B R</t>
+          <t>Head 24L B G</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp R; was with 24L T on OU2</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was with 24L T on OU2</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4695,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Head 34L T G</t>
+          <t>Head 34L T R</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4715,7 +4715,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -4725,7 +4725,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C2 235</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was was C2 235</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Head 34L T R</t>
+          <t>Head 34L T G</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4859,7 +4859,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -4869,7 +4869,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was was C2 235</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C2 235</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Head 34L B G</t>
+          <t>Head 34L B R</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4931,7 +4931,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 34L T on OU2</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 34L T on OU2</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5055,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Head 34L B R</t>
+          <t>Head 34L B G</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -5075,7 +5075,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -5085,7 +5085,7 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 34L T on OU2</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 34L T on OU2</t>
         </is>
       </c>
     </row>
@@ -5127,7 +5127,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Head 32R G</t>
+          <t>Head 32R R</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G with 34L; Y/R on 34R OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was R with 34L; Y/G on 34R OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -5229,7 +5229,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was G with 34L; Y/R on 34R OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was R with 34L; Y/G on 34R OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Head 32R R</t>
+          <t>Head 32R G</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -5301,7 +5301,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was G with 34L; Y/R on 34R OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was R with 34L; Y/G on 34R OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Head 34R T G</t>
+          <t>Head 34R T R</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -5373,7 +5373,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was was C2 237</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was was C2 237</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5487,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Head 34R T R</t>
+          <t>Head 34R T G</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -5517,7 +5517,7 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was was C2 237</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was was C2 237</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5559,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Head 34R B G</t>
+          <t>Head 34R B R</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5579,7 +5579,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -5589,7 +5589,7 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was with 34R T on OU3</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was with 34R T on OU3</t>
         </is>
       </c>
     </row>
@@ -5703,7 +5703,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Head 34R B R</t>
+          <t>Head 34R B G</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -5733,7 +5733,7 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was with 34R T on OU3</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was with 34R T on OU3</t>
         </is>
       </c>
     </row>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Head 36RA T G</t>
+          <t>Head 36RA T R</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -5805,7 +5805,7 @@
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was S1-2 G/Y/R</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was S1-2 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -5877,7 +5877,7 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp Y; was S1-2 G/Y/R</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp Y; was S1-2 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -5919,7 +5919,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Head 36RA T R</t>
+          <t>Head 36RA T G</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was S1-2 G/Y/R</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was S1-2 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -5991,7 +5991,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Head 36RA B G</t>
+          <t>Head 36RA B R</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -6011,7 +6011,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -6021,7 +6021,7 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was with 36RA T on OU2</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was with 36RA T on OU2</t>
         </is>
       </c>
     </row>
@@ -6135,7 +6135,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Head 36RA B R</t>
+          <t>Head 36RA B G</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -6155,7 +6155,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was with 36RA T on OU2</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was with 36RA T on OU2</t>
         </is>
       </c>
     </row>
@@ -6207,7 +6207,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Head 36RB T G</t>
+          <t>Head 36RB T R</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C11 1132</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was was C11 1132</t>
         </is>
       </c>
     </row>
@@ -6351,7 +6351,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Head 36RB T R</t>
+          <t>Head 36RB T G</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
@@ -6381,7 +6381,7 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was was C11 1132</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C11 1132</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6423,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Head 36RB B G</t>
+          <t>Head 36RB B R</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
@@ -6453,7 +6453,7 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 36RB T on OU3</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 36RB T on OU3</t>
         </is>
       </c>
     </row>
@@ -6567,7 +6567,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Head 36RB B R</t>
+          <t>Head 36RB B G</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -6587,7 +6587,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -6597,7 +6597,7 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 36RB T on OU3</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 36RB T on OU3</t>
         </is>
       </c>
     </row>
@@ -6639,7 +6639,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Head 38LB T G</t>
+          <t>Head 38LB T R</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6659,7 +6659,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -6669,7 +6669,7 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was S1-3 G/Y/R</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp R; was S1-3 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -6741,7 +6741,7 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp Y; was S1-3 G/Y/R</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp Y; was S1-3 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -6783,7 +6783,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Head 38LB T R</t>
+          <t>Head 38LB T G</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
@@ -6813,7 +6813,7 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp R; was S1-3 G/Y/R</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was S1-3 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Head 38LB B G</t>
+          <t>Head 38LB B R</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6875,7 +6875,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
@@ -6885,7 +6885,7 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>LCOS Signal 8 UID 40; STOP/APPROACH/CLEAR; lamp G; was with 38LB T on OU4</t>
+          <t>LCOS Signal 8 UID 40; STOP/APPROACH/CLEAR; lamp R; was with 38LB T on OU4</t>
         </is>
       </c>
     </row>
@@ -6999,7 +6999,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Head 38LB B R</t>
+          <t>Head 38LB B G</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -7019,7 +7019,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M92" t="inlineStr">
@@ -7029,7 +7029,7 @@
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>LCOS Signal 8 UID 40; STOP/APPROACH/CLEAR; lamp R; was with 38LB T on OU4</t>
+          <t>LCOS Signal 8 UID 40; STOP/APPROACH/CLEAR; lamp G; was with 38LB T on OU4</t>
         </is>
       </c>
     </row>
@@ -7071,7 +7071,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Head 38LA G</t>
+          <t>Head 38LA R</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -7091,7 +7091,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
@@ -7101,7 +7101,7 @@
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp G; was leftover trio on 36 boards; 38LB keeps OU4</t>
+          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp R; was leftover trio on 36 boards; 38LB keeps OU4</t>
         </is>
       </c>
     </row>
@@ -7215,7 +7215,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Head 38LA R</t>
+          <t>Head 38LA G</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -7235,7 +7235,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
@@ -7245,7 +7245,7 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp R; was leftover trio on 36 boards; 38LB keeps OU4</t>
+          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp G; was leftover trio on 36 boards; 38LB keeps OU4</t>
         </is>
       </c>
     </row>
@@ -7287,7 +7287,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Head 40LB T G</t>
+          <t>Head 40LB T R</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -7307,7 +7307,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C1 132</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was was C1 132</t>
         </is>
       </c>
     </row>
@@ -7431,7 +7431,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Head 40LB T R</t>
+          <t>Head 40LB T G</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -7451,7 +7451,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
@@ -7461,7 +7461,7 @@
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was was C1 132</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C1 132</t>
         </is>
       </c>
     </row>
@@ -7503,7 +7503,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Head 40LB B G</t>
+          <t>Head 40LB B R</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -7523,7 +7523,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was with 40LB T on OU2</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was with 40LB T on OU2</t>
         </is>
       </c>
     </row>
@@ -7647,7 +7647,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Head 40LB B R</t>
+          <t>Head 40LB B G</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -7667,7 +7667,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M101" t="inlineStr">
@@ -7677,7 +7677,7 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was with 40LB T on OU2</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was with 40LB T on OU2</t>
         </is>
       </c>
     </row>
@@ -7719,7 +7719,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>Head 40LA G</t>
+          <t>Head 40LA R</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -7739,7 +7739,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M102" t="inlineStr">
@@ -7749,7 +7749,7 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was whole dwarf on OU3; 2035/2036 can sit apart</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was whole dwarf on OU3; 2035/2036 can sit apart</t>
         </is>
       </c>
     </row>
@@ -7863,7 +7863,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Head 40LA R</t>
+          <t>Head 40LA G</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7883,7 +7883,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M104" t="inlineStr">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was whole dwarf on OU3; 2035/2036 can sit apart</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was whole dwarf on OU3; 2035/2036 can sit apart</t>
         </is>
       </c>
     </row>
@@ -7935,7 +7935,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Head 2036 G</t>
+          <t>Head 2036 R</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7955,7 +7955,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M105" t="inlineStr">
@@ -7965,7 +7965,7 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was balloon; sequential G/Y/R</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was balloon; sequential R/Y/G</t>
         </is>
       </c>
     </row>
@@ -8037,7 +8037,7 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp Y; was balloon; sequential G/Y/R</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp Y; was balloon; sequential R/Y/G</t>
         </is>
       </c>
     </row>
@@ -8079,7 +8079,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Head 2036 R</t>
+          <t>Head 2036 G</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -8099,7 +8099,7 @@
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M107" t="inlineStr">
@@ -8109,7 +8109,7 @@
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was balloon; sequential G/Y/R</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was balloon; sequential R/Y/G</t>
         </is>
       </c>
     </row>
@@ -8151,7 +8151,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>Head 2035 G</t>
+          <t>Head 2035 R</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M108" t="inlineStr">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was leftover trio (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was leftover trio (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -8295,7 +8295,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Head 2035 R</t>
+          <t>Head 2035 G</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -8315,7 +8315,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M110" t="inlineStr">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was leftover trio (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was leftover trio (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -8411,7 +8411,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -8421,7 +8421,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH432)(IH433)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH432)(IH433)</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -8463,7 +8463,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH434)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH434)</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -8515,7 +8515,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -8525,7 +8525,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH438)(IH439)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH438)(IH439)</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -8567,7 +8567,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH436)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH436)</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -8619,7 +8619,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -8629,7 +8629,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH437)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH437)</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -8681,7 +8681,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1332)(IH1333)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH1332)(IH1333)</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -8723,7 +8723,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1335)(IH1336)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH1335)(IH1336)</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -8775,7 +8775,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -8785,7 +8785,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1337)(IH1338)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH1337)(IH1338)</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -8827,7 +8827,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -8837,7 +8837,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1334)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH1334)</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -8889,7 +8889,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH232)(IH238)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH232)(IH238)</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -8931,7 +8931,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -8941,7 +8941,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH234)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH234)</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -8983,7 +8983,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH233)(IH239)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH233)(IH239)</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -9035,7 +9035,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -9045,7 +9045,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1232)(IH1233)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH1232)(IH1233)</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -9087,7 +9087,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -9097,7 +9097,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1234)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH1234)</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -9139,7 +9139,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -9149,7 +9149,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1235)(IH1236)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH1235)(IH1236)</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -9201,7 +9201,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH135)(IH136)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH135)(IH136)</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -9253,7 +9253,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH132)(IH133)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH132)(IH133)</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -9295,7 +9295,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -9305,7 +9305,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH139)(IH140)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH139)(IH140)</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -9347,7 +9347,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH143)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH143)</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -9399,7 +9399,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -9409,7 +9409,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1132)(IH1135)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH1132)(IH1135)</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -9451,7 +9451,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -9461,7 +9461,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1136)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH1136)</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -9513,7 +9513,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1133)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH1133)</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -9555,7 +9555,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -9565,7 +9565,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1134)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH1134)</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -11914,7 +11914,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Head 36RA T G</t>
+          <t>Head 36RA T R</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -11929,7 +11929,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/135; packed 135 (node 1 sig 3); was S1-1 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/135; packed 135 (node 1 sig 3); was S1-1 G</t>
         </is>
       </c>
     </row>
@@ -11994,7 +11994,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Head 36RA T R</t>
+          <t>Head 36RA T G</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -12009,7 +12009,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/135; packed 135 (node 1 sig 3); was S1-1 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/135; packed 135 (node 1 sig 3); was S1-1 R</t>
         </is>
       </c>
     </row>
@@ -12034,7 +12034,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Head 36RA B G</t>
+          <t>Head 36RA B R</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -12049,7 +12049,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/136; packed 136 (node 1 sig 4); was S1-2 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/136; packed 136 (node 1 sig 4); was S1-2 G</t>
         </is>
       </c>
     </row>
@@ -12114,7 +12114,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Head 36RA B R</t>
+          <t>Head 36RA B G</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -12129,7 +12129,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/136; packed 136 (node 1 sig 4); was S1-2 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/136; packed 136 (node 1 sig 4); was S1-2 R</t>
         </is>
       </c>
     </row>
@@ -12154,7 +12154,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Head 38LA R</t>
+          <t>Head 38LA G</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -12169,7 +12169,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/143; packed 143 (node 1 sig 11)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/143; packed 143 (node 1 sig 11)</t>
         </is>
       </c>
     </row>
@@ -12234,7 +12234,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Head 36RB T G</t>
+          <t>Head 36RB T R</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -12249,7 +12249,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/132; packed 132 (node 1 sig 0); was S1-3 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/132; packed 132 (node 1 sig 0); was S1-3 G</t>
         </is>
       </c>
     </row>
@@ -12314,7 +12314,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Head 36RB T R</t>
+          <t>Head 36RB T G</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -12329,7 +12329,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/132; packed 132 (node 1 sig 0); was S1-3 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/132; packed 132 (node 1 sig 0); was S1-3 R</t>
         </is>
       </c>
     </row>
@@ -12354,7 +12354,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Head 36RB B G</t>
+          <t>Head 36RB B R</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -12369,7 +12369,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/133; packed 133 (node 1 sig 1); was S1-4 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/133; packed 133 (node 1 sig 1); was S1-4 G</t>
         </is>
       </c>
     </row>
@@ -12434,7 +12434,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Head 36RB B R</t>
+          <t>Head 36RB B G</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -12449,7 +12449,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/133; packed 133 (node 1 sig 1); was S1-4 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/133; packed 133 (node 1 sig 1); was S1-4 R</t>
         </is>
       </c>
     </row>
@@ -12474,7 +12474,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Head 38LA G</t>
+          <t>Head 38LA R</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -12489,7 +12489,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/143; packed 143 (node 1 sig 11)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/143; packed 143 (node 1 sig 11)</t>
         </is>
       </c>
     </row>
@@ -12874,7 +12874,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Head 34L T G</t>
+          <t>Head 34L T R</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -12889,7 +12889,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1232; packed 1232 (node 12 sig 0); was S2-1 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1232; packed 1232 (node 12 sig 0); was S2-1 G</t>
         </is>
       </c>
     </row>
@@ -12954,7 +12954,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Head 34L T R</t>
+          <t>Head 34L T G</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -12969,7 +12969,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1232; packed 1232 (node 12 sig 0); was S2-1 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1232; packed 1232 (node 12 sig 0); was S2-1 R</t>
         </is>
       </c>
     </row>
@@ -12994,7 +12994,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Head 34L B G</t>
+          <t>Head 34L B R</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -13009,7 +13009,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1233; packed 1233 (node 12 sig 1); was S2-2 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1233; packed 1233 (node 12 sig 1); was S2-2 G</t>
         </is>
       </c>
     </row>
@@ -13074,7 +13074,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Head 34L B R</t>
+          <t>Head 34L B G</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -13089,7 +13089,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1233; packed 1233 (node 12 sig 1); was S2-2 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1233; packed 1233 (node 12 sig 1); was S2-2 R</t>
         </is>
       </c>
     </row>
@@ -13114,7 +13114,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Head 32R G</t>
+          <t>Head 32R R</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -13129,7 +13129,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1234; packed 1234 (node 12 sig 2); was S2-8 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1234; packed 1234 (node 12 sig 2); was S2-8 Y</t>
         </is>
       </c>
     </row>
@@ -13194,7 +13194,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Head 34R T G</t>
+          <t>Head 34R T R</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -13209,7 +13209,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1235; packed 1235 (node 12 sig 3); was S2-9 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1235; packed 1235 (node 12 sig 3); was S2-9 G</t>
         </is>
       </c>
     </row>
@@ -13274,7 +13274,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Head 34R T R</t>
+          <t>Head 34R T G</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -13289,7 +13289,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1235; packed 1235 (node 12 sig 3); was S2-9 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1235; packed 1235 (node 12 sig 3); was S2-9 Y</t>
         </is>
       </c>
     </row>
@@ -13314,7 +13314,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Head 34R B G</t>
+          <t>Head 34R B R</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -13329,7 +13329,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1236; packed 1236 (node 12 sig 4); was S2-4 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1236; packed 1236 (node 12 sig 4); was S2-4 G</t>
         </is>
       </c>
     </row>
@@ -13394,7 +13394,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Head 34R B R</t>
+          <t>Head 34R B G</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -13409,7 +13409,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1236; packed 1236 (node 12 sig 4); was S2-4 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1236; packed 1236 (node 12 sig 4); was S2-4 R</t>
         </is>
       </c>
     </row>
@@ -13434,7 +13434,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Head 32R R</t>
+          <t>Head 32R G</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -13449,7 +13449,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1234; packed 1234 (node 12 sig 2); was S2-8 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1234; packed 1234 (node 12 sig 2); was S2-8 G</t>
         </is>
       </c>
     </row>
@@ -13514,7 +13514,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Head 24RA T G</t>
+          <t>Head 24RA T R</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -13529,7 +13529,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/232; packed 232 (node 2 sig 0)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/232; packed 232 (node 2 sig 0)</t>
         </is>
       </c>
     </row>
@@ -13594,7 +13594,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Head 24RA T R</t>
+          <t>Head 24RA T G</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -13609,7 +13609,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/232; packed 232 (node 2 sig 0)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/232; packed 232 (node 2 sig 0)</t>
         </is>
       </c>
     </row>
@@ -13634,7 +13634,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Head 24RA B G</t>
+          <t>Head 24RA B R</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -13649,7 +13649,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/238; packed 238 (node 2 sig 6)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/238; packed 238 (node 2 sig 6)</t>
         </is>
       </c>
     </row>
@@ -13714,7 +13714,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Head 24RA B R</t>
+          <t>Head 24RA B G</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -13729,7 +13729,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/238; packed 238 (node 2 sig 6)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/238; packed 238 (node 2 sig 6)</t>
         </is>
       </c>
     </row>
@@ -13824,7 +13824,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Head 24L T G</t>
+          <t>Head 24L T R</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -13839,7 +13839,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/233; packed 233 (node 2 sig 1); was S2-5 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/233; packed 233 (node 2 sig 1); was S2-5 G</t>
         </is>
       </c>
     </row>
@@ -13904,7 +13904,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Head 24L T R</t>
+          <t>Head 24L T G</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -13919,7 +13919,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/233; packed 233 (node 2 sig 1); was S2-5 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/233; packed 233 (node 2 sig 1); was S2-5 R</t>
         </is>
       </c>
     </row>
@@ -13944,7 +13944,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Head 24L B G</t>
+          <t>Head 24L B R</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -13959,7 +13959,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/239; packed 239 (node 2 sig 7); was S2-3 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/239; packed 239 (node 2 sig 7); was S2-3 G</t>
         </is>
       </c>
     </row>
@@ -14024,7 +14024,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Head 24L B R</t>
+          <t>Head 24L B G</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -14039,7 +14039,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/239; packed 239 (node 2 sig 7); was S2-3 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/239; packed 239 (node 2 sig 7); was S2-3 R</t>
         </is>
       </c>
     </row>
@@ -14279,7 +14279,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Head 24RB G</t>
+          <t>Head 24RB R</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -14294,7 +14294,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
         </is>
       </c>
     </row>
@@ -14359,7 +14359,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Head 24RB R</t>
+          <t>Head 24RB G</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -14374,7 +14374,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
         </is>
       </c>
     </row>
@@ -14969,7 +14969,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Head 8RA T G</t>
+          <t>Head 8RA T R</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -14984,7 +14984,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1332; packed 1332 (node 13 sig 0); was S3-10 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1332; packed 1332 (node 13 sig 0); was S3-10 G</t>
         </is>
       </c>
     </row>
@@ -15049,7 +15049,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Head 8RA T R</t>
+          <t>Head 8RA T G</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -15064,7 +15064,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1332; packed 1332 (node 13 sig 0); was S3-10 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1332; packed 1332 (node 13 sig 0); was S3-10 R</t>
         </is>
       </c>
     </row>
@@ -15089,7 +15089,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Head 8RA B G</t>
+          <t>Head 8RA B R</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -15104,7 +15104,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1333; packed 1333 (node 13 sig 1); was S3-12 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1333; packed 1333 (node 13 sig 1); was S3-12 G</t>
         </is>
       </c>
     </row>
@@ -15169,7 +15169,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Head 8RA B R</t>
+          <t>Head 8RA B G</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1333; packed 1333 (node 13 sig 1); was S3-12 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1333; packed 1333 (node 13 sig 1); was S3-12 Y</t>
         </is>
       </c>
     </row>
@@ -15279,7 +15279,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Head 8LA T G</t>
+          <t>Head 8LA T R</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -15294,7 +15294,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 G</t>
         </is>
       </c>
     </row>
@@ -15359,7 +15359,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Head 8LA T R</t>
+          <t>Head 8LA T G</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -15374,7 +15374,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 R</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Head 8LA B G</t>
+          <t>Head 8LA B R</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -15414,7 +15414,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 G</t>
         </is>
       </c>
     </row>
@@ -15479,7 +15479,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Head 8LA B R</t>
+          <t>Head 8LA B G</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -15494,7 +15494,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 R</t>
         </is>
       </c>
     </row>
@@ -15519,7 +15519,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Head 8LB G</t>
+          <t>Head 8LB R</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -15534,7 +15534,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2); was S3-14 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2); was S3-14 Y</t>
         </is>
       </c>
     </row>
@@ -15919,7 +15919,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Head 6LB T G</t>
+          <t>Head 6LB T R</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -15934,7 +15934,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/432; packed 432 (node 4 sig 0); was S3-1 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/432; packed 432 (node 4 sig 0); was S3-1 G</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Head 6LB T R</t>
+          <t>Head 6LB T G</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -16014,7 +16014,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/432; packed 432 (node 4 sig 0); was S3-1 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/432; packed 432 (node 4 sig 0); was S3-1 R</t>
         </is>
       </c>
     </row>
@@ -16039,7 +16039,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Head 6LB B G</t>
+          <t>Head 6LB B R</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -16054,7 +16054,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/433; packed 433 (node 4 sig 1); was S3-13 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/433; packed 433 (node 4 sig 1); was S3-13 G</t>
         </is>
       </c>
     </row>
@@ -16119,7 +16119,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Head 6LB B R</t>
+          <t>Head 6LB B G</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -16134,7 +16134,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/433; packed 433 (node 4 sig 1); was S3-13 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/433; packed 433 (node 4 sig 1); was S3-13 Y</t>
         </is>
       </c>
     </row>
@@ -16159,7 +16159,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Head 6LA G</t>
+          <t>Head 6LA R</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -16174,7 +16174,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/434; packed 434 (node 4 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/434; packed 434 (node 4 sig 2)</t>
         </is>
       </c>
     </row>
@@ -16239,7 +16239,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Head 2L T G</t>
+          <t>Head 2L T R</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -16254,7 +16254,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/438; packed 438 (node 4 sig 6); was S3-2 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/438; packed 438 (node 4 sig 6); was S3-2 G</t>
         </is>
       </c>
     </row>
@@ -16319,7 +16319,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Head 2L T R</t>
+          <t>Head 2L T G</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -16334,7 +16334,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/438; packed 438 (node 4 sig 6); was S3-2 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/438; packed 438 (node 4 sig 6); was S3-2 R</t>
         </is>
       </c>
     </row>
@@ -16359,7 +16359,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Head 2L B G</t>
+          <t>Head 2L B R</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -16374,7 +16374,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/439; packed 439 (node 4 sig 7); was S3-3 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/439; packed 439 (node 4 sig 7); was S3-3 G</t>
         </is>
       </c>
     </row>
@@ -16439,7 +16439,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Head 2L B R</t>
+          <t>Head 2L B G</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -16454,7 +16454,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/439; packed 439 (node 4 sig 7); was S3-3 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/439; packed 439 (node 4 sig 7); was S3-3 R</t>
         </is>
       </c>
     </row>
@@ -16479,7 +16479,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Head 6LA R</t>
+          <t>Head 6LA G</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -16494,7 +16494,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/434; packed 434 (node 4 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/434; packed 434 (node 4 sig 2)</t>
         </is>
       </c>
     </row>
@@ -16849,7 +16849,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Head 40LB T G</t>
+          <t>Head 40LB T R</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -16864,7 +16864,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1132; packed 1132 (node 11 sig 0); was S1-5 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1132; packed 1132 (node 11 sig 0); was S1-5 G</t>
         </is>
       </c>
     </row>
@@ -16929,7 +16929,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Head 40LB T R</t>
+          <t>Head 40LB T G</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -16944,7 +16944,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1132; packed 1132 (node 11 sig 0); was S1-5 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1132; packed 1132 (node 11 sig 0); was S1-5 Y</t>
         </is>
       </c>
     </row>
@@ -16969,7 +16969,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Head 40LB B G</t>
+          <t>Head 40LB B R</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -16984,7 +16984,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1135; packed 1135 (node 11 sig 3); was S1-6 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1135; packed 1135 (node 11 sig 3); was S1-6 G</t>
         </is>
       </c>
     </row>
@@ -17049,7 +17049,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Head 40LB B R</t>
+          <t>Head 40LB B G</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -17064,7 +17064,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1135; packed 1135 (node 11 sig 3); was S1-6 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1135; packed 1135 (node 11 sig 3); was S1-6 Y</t>
         </is>
       </c>
     </row>
@@ -17089,7 +17089,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Head 2035 R</t>
+          <t>Head 2035 G</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -17104,7 +17104,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2)</t>
         </is>
       </c>
     </row>
@@ -17169,7 +17169,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Head 40LA G</t>
+          <t>Head 40LA R</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -17184,7 +17184,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4); was S4-6 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4); was S4-6 G</t>
         </is>
       </c>
     </row>
@@ -17249,7 +17249,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Head 40LA R</t>
+          <t>Head 40LA G</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -17264,7 +17264,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4); was S4-6 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4); was S4-6 Y</t>
         </is>
       </c>
     </row>
@@ -17289,7 +17289,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Head 2036 G</t>
+          <t>Head 2036 R</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -17304,7 +17304,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-7 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-7 G</t>
         </is>
       </c>
     </row>
@@ -17369,7 +17369,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Head 2036 R</t>
+          <t>Head 2036 G</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -17384,7 +17384,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-7 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-7 Y</t>
         </is>
       </c>
     </row>
@@ -17409,7 +17409,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Head 2035 G</t>
+          <t>Head 2035 R</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -17424,7 +17424,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2)</t>
         </is>
       </c>
     </row>
@@ -23239,7 +23239,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>Head 38LB T G</t>
+          <t>Head 38LB T R</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
@@ -23254,7 +23254,7 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/139; packed 139 (node 1 sig 7)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/139; packed 139 (node 1 sig 7)</t>
         </is>
       </c>
     </row>
@@ -23319,7 +23319,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Head 38LB T R</t>
+          <t>Head 38LB T G</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
@@ -23334,7 +23334,7 @@
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/139; packed 139 (node 1 sig 7)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/139; packed 139 (node 1 sig 7)</t>
         </is>
       </c>
     </row>
@@ -23359,7 +23359,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Head 38LB B G</t>
+          <t>Head 38LB B R</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
@@ -23374,7 +23374,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/140; packed 140 (node 1 sig 8)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/140; packed 140 (node 1 sig 8)</t>
         </is>
       </c>
     </row>
@@ -23439,7 +23439,7 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Head 38LB B R</t>
+          <t>Head 38LB B G</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
@@ -23454,7 +23454,7 @@
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/140; packed 140 (node 1 sig 8)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/140; packed 140 (node 1 sig 8)</t>
         </is>
       </c>
     </row>
@@ -23539,7 +23539,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Head 4RA G</t>
+          <t>Head 4RA R</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -23554,7 +23554,7 @@
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/436; packed 436 (node 4 sig 4)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/436; packed 436 (node 4 sig 4)</t>
         </is>
       </c>
     </row>
@@ -23619,7 +23619,7 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Head 4RA R</t>
+          <t>Head 4RA G</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
@@ -23634,7 +23634,7 @@
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/436; packed 436 (node 4 sig 4)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/436; packed 436 (node 4 sig 4)</t>
         </is>
       </c>
     </row>
@@ -23659,7 +23659,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>Head 4RB G</t>
+          <t>Head 4RB R</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
@@ -23674,7 +23674,7 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/437; packed 437 (node 4 sig 5)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/437; packed 437 (node 4 sig 5)</t>
         </is>
       </c>
     </row>
@@ -23739,7 +23739,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Head 4RB R</t>
+          <t>Head 4RB G</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
@@ -23754,7 +23754,7 @@
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/437; packed 437 (node 4 sig 5)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/437; packed 437 (node 4 sig 5)</t>
         </is>
       </c>
     </row>
@@ -23839,7 +23839,7 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Head 8RB T G</t>
+          <t>Head 8RB T R</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
@@ -23854,7 +23854,7 @@
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1335; packed 1335 (node 13 sig 3)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1335; packed 1335 (node 13 sig 3)</t>
         </is>
       </c>
     </row>
@@ -23919,7 +23919,7 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Head 8RB T R</t>
+          <t>Head 8RB T G</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
@@ -23934,7 +23934,7 @@
       </c>
       <c r="H324" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1335; packed 1335 (node 13 sig 3)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1335; packed 1335 (node 13 sig 3)</t>
         </is>
       </c>
     </row>
@@ -23959,7 +23959,7 @@
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Head 8RB B G</t>
+          <t>Head 8RB B R</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
@@ -23974,7 +23974,7 @@
       </c>
       <c r="H325" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1336; packed 1336 (node 13 sig 4)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1336; packed 1336 (node 13 sig 4)</t>
         </is>
       </c>
     </row>
@@ -24039,7 +24039,7 @@
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Head 8RB B R</t>
+          <t>Head 8RB B G</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
@@ -24054,7 +24054,7 @@
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1336; packed 1336 (node 13 sig 4)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1336; packed 1336 (node 13 sig 4)</t>
         </is>
       </c>
     </row>
@@ -24079,7 +24079,7 @@
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Head 8LB R</t>
+          <t>Head 8LB G</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
@@ -24094,7 +24094,7 @@
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2)</t>
         </is>
       </c>
     </row>
@@ -29562,17 +29562,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>C1-OU2-1</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>C1-OU2-2</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>C1-OU2-3</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>C1-OU2-2</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>C1-OU2-1</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -29654,17 +29654,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>C11-OU3-4</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>C11-OU3-5</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
           <t>C11-OU3-6</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>C11-OU3-5</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>C11-OU3-4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -29751,17 +29751,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>C11-OU3-7</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>C11-OU3-8</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
           <t>C11-OU2-7</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>C11-OU3-8</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>C11-OU3-7</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -29930,17 +29930,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>C2-OU2-1</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>C2-OU2-2</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t>C2-OU2-3</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>C2-OU2-2</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>C2-OU2-1</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -30027,17 +30027,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>C12-OU2-1</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>C12-OU2-2</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
           <t>C12-OU2-3</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>C12-OU2-2</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>C12-OU2-1</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -30141,17 +30141,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>C12-OU2-7</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>C12-OU3-8</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
           <t>C12-OU3-7</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>C12-OU3-8</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>C12-OU2-7</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -30558,17 +30558,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
+          <t>C4-OU3-1</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>C4-OU3-2</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
           <t>C4-OU3-3</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>C4-OU3-2</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>C4-OU3-1</t>
         </is>
       </c>
     </row>
@@ -30677,17 +30677,17 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
+          <t>C4-OU2-7</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>C4-OU3-8</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
           <t>C4-OU3-7</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>C4-OU3-8</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>C4-OU2-7</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -31547,17 +31547,17 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
+          <t>C13-OU1-1</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>C13-OU1-2</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
           <t>C13-OU1-3</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>C13-OU1-2</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>C13-OU1-1</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">

</xml_diff>

<commit_message>
Commission Barn/EH turnout FB and move C13 motors to OU2.
Switch 7/11/13 are TWOSENSOR (Pi tables); Switch 7/9/11 motors sit on C13-OU2 with Digicon 8LA/8LB moved to OU3. Wiring inventory and Signal Manager plan updated.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
+++ b/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
@@ -2932,7 +2932,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>C13-OU2-1</t>
+          <t>C13-OU3-1</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3004,7 +3004,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>C13-OU2-2</t>
+          <t>C13-OU3-2</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3076,7 +3076,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>C13-OU2-3</t>
+          <t>C13-OU3-3</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3148,7 +3148,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>C13-OU2-4</t>
+          <t>C13-OU3-4</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3213,14 +3213,14 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was with 8LA T on OU2</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was with 8LA T on OU3</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>C13-OU2-5</t>
+          <t>C13-OU3-5</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3285,14 +3285,14 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp Y; was with 8LA T on OU2</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp Y; was with 8LA T on OU3</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>C13-OU2-6</t>
+          <t>C13-OU3-6</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3357,14 +3357,14 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was with 8LA T on OU2</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was with 8LA T on OU3</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>C13-OU2-7</t>
+          <t>C13-OU3-7</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3429,14 +3429,14 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was R/Y with 8LA; G spills to 8RB OU4</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was R/Y with 8LA on OU3; G spills to 8RB OU4</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>C13-OU2-8</t>
+          <t>C13-OU3-8</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3501,7 +3501,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was R/Y with 8LA; G spills to 8RB OU4</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was R/Y with 8LA on OU3; G spills to 8RB OU4</t>
         </is>
       </c>
     </row>
@@ -8800,7 +8800,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>C13-OU2-1 C13-OU2-2 C13-OU2-3 C13-OU2-4 C13-OU2-5 C13-OU2-6</t>
+          <t>C13-OU3-1 C13-OU3-2 C13-OU3-3 C13-OU3-4 C13-OU3-5 C13-OU3-6</t>
         </is>
       </c>
     </row>
@@ -8852,7 +8852,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>C13-OU2-7 C13-OU2-8 C13-OU4-7</t>
+          <t>C13-OU3-7 C13-OU3-8 C13-OU4-7</t>
         </is>
       </c>
     </row>
@@ -10725,6 +10725,11 @@
       <c r="M10" t="n">
         <v>3</v>
       </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>C13-OU2-1, C13-OU2-2, C13-OU2-3, C13-OU2-4, C13-OU2-5, C13-OU2-6</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr">
         <is>
           <t>Switch 7, Switch 11, Switch 9</t>
@@ -10772,7 +10777,7 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>8RA, 8LA, 8LB, 8RB</t>
+          <t>8RA, S3-4, S3-5, S3-14, 8LA, 8LB, 8RB</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
@@ -15271,7 +15276,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -15279,22 +15284,22 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Head 8LA T R</t>
+          <t>Switch 7 N</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Turnout Motor</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 G</t>
+          <t>radio 13 | M2T1308 / Node: 13 Turnout: 0 | DCC 117 | ports 1,2</t>
         </is>
       </c>
     </row>
@@ -15311,7 +15316,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -15319,22 +15324,22 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Head 8LA T Y</t>
+          <t>Switch 7 R</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Turnout Motor</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 Y</t>
+          <t>radio 13 | M2T1308 / Node: 13 Turnout: 0 | DCC 117 | ports 1,2</t>
         </is>
       </c>
     </row>
@@ -15351,7 +15356,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -15359,22 +15364,22 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Head 8LA T G</t>
+          <t>Switch 11 N</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Turnout Motor</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 R</t>
+          <t>radio 13 | M2T1309 / Node: 13 Turnout: 1 | DCC 118 | ports 3,4</t>
         </is>
       </c>
     </row>
@@ -15391,7 +15396,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -15399,22 +15404,22 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Head 8LA B R</t>
+          <t>Switch 11 R</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Turnout Motor</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 G</t>
+          <t>radio 13 | M2T1309 / Node: 13 Turnout: 1 | DCC 118 | ports 3,4</t>
         </is>
       </c>
     </row>
@@ -15431,7 +15436,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -15439,22 +15444,22 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Head 8LA B Y</t>
+          <t>Switch 9 N</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Turnout Motor</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 Y</t>
+          <t>radio 13 | M2T1310 / Node: 13 Turnout: 2 | DCC 119 | ports 5,6</t>
         </is>
       </c>
     </row>
@@ -15471,7 +15476,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -15479,22 +15484,22 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Head 8LA B G</t>
+          <t>Switch 9 R</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Turnout Motor</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 R</t>
+          <t>radio 13 | M2T1310 / Node: 13 Turnout: 2 | DCC 119 | ports 5,6</t>
         </is>
       </c>
     </row>
@@ -15511,30 +15516,20 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D104" t="n">
         <v>7</v>
       </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>Head 8LB R</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>Searchlight Signal Head</t>
-        </is>
-      </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2); was S3-14 Y</t>
+          <t>spare (was leftover S3 RGB; motors use 1–6)</t>
         </is>
       </c>
     </row>
@@ -15551,30 +15546,20 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D105" t="n">
         <v>8</v>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>Head 8LB Y</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>Searchlight Signal Head</t>
-        </is>
-      </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2)</t>
+          <t>spare</t>
         </is>
       </c>
     </row>
@@ -22651,7 +22636,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -22659,22 +22644,22 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>Switch 7 N</t>
+          <t>Head 8LA T R</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>Turnout Motor</t>
+          <t>Searchlight Signal Head</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>radio addr 13 | M2T1308 / switch_id 13-8 / DCC 117 | TO6; TO8 shares motor (IT37) | ASSUMED on new C13-OU3 12V board — confirm physical board ID</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5)</t>
         </is>
       </c>
     </row>
@@ -22691,7 +22676,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -22699,22 +22684,22 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>Switch 7 R</t>
+          <t>Head 8LA T Y</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>Turnout Motor</t>
+          <t>Searchlight Signal Head</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>radio addr 13 | M2T1308 / switch_id 13-8 / DCC 117 | TO6 | ASSUMED on new C13-OU3 12V board — confirm physical board ID</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5)</t>
         </is>
       </c>
     </row>
@@ -22731,7 +22716,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D292" t="n">
@@ -22739,22 +22724,22 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>Switch 11 N</t>
+          <t>Head 8LA T G</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>Turnout Motor</t>
+          <t>Searchlight Signal Head</t>
         </is>
       </c>
       <c r="G292" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>radio addr 13 | M2T1309 / switch_id 13-9 / DCC 118 | TO11 | ASSUMED on new C13-OU3 12V board — confirm physical board ID</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5)</t>
         </is>
       </c>
     </row>
@@ -22771,7 +22756,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D293" t="n">
@@ -22779,22 +22764,22 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Switch 11 R</t>
+          <t>Head 8LA B R</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>Turnout Motor</t>
+          <t>Searchlight Signal Head</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>radio addr 13 | M2T1309 / switch_id 13-9 / DCC 118 | TO11 | ASSUMED on new C13-OU3 12V board — confirm physical board ID</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6)</t>
         </is>
       </c>
     </row>
@@ -22811,7 +22796,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D294" t="n">
@@ -22819,22 +22804,22 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Switch 9 N</t>
+          <t>Head 8LA B Y</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>Turnout Motor</t>
+          <t>Searchlight Signal Head</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>radio addr 13 | M2T1310 / switch_id 13-10 / DCC 119 | TO10 | ASSUMED on new C13-OU3 12V board — confirm physical board ID</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6)</t>
         </is>
       </c>
     </row>
@@ -22851,7 +22836,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D295" t="n">
@@ -22859,22 +22844,22 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Switch 9 R</t>
+          <t>Head 8LA B G</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>Turnout Motor</t>
+          <t>Searchlight Signal Head</t>
         </is>
       </c>
       <c r="G295" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>radio addr 13 | M2T1310 / switch_id 13-10 / DCC 119 | TO10 | ASSUMED on new C13-OU3 12V board — confirm physical board ID</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6)</t>
         </is>
       </c>
     </row>
@@ -22891,20 +22876,30 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D296" t="n">
         <v>7</v>
       </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Head 8LB R</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Searchlight Signal Head</t>
+        </is>
+      </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>free | C13-OU3 12V</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2)</t>
         </is>
       </c>
     </row>
@@ -22921,20 +22916,30 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D297" t="n">
         <v>8</v>
       </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Head 8LB Y</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Searchlight Signal Head</t>
+        </is>
+      </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>free | C13-OU3 12V</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2)</t>
         </is>
       </c>
     </row>
@@ -28545,7 +28550,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>M2S1367 / Switch 13-1 FB N | ASSUMED on new C13-IN1 — confirm physical board ID</t>
+          <t>M2S1367 / Switch 13-1 FB N | commissioned 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -28580,7 +28585,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>M2S1368 / Switch 13-1 FB R | ASSUMED on new C13-IN1 — confirm physical board ID</t>
+          <t>M2S1368 / Switch 13-1 FB R | commissioned 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -28615,7 +28620,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>M2S1369 / Switch 13-2 FB N | ASSUMED on new C13-IN1 — confirm physical board ID</t>
+          <t>M2S1369 / Switch 13-2 FB N | commissioned 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -28650,7 +28655,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>M2S1370 / Switch 13-2 FB R | ASSUMED on new C13-IN1 — confirm physical board ID</t>
+          <t>M2S1370 / Switch 13-2 FB R | commissioned 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -28685,7 +28690,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>M2S1371 / Switch 13-3 FB N | ASSUMED on new C13-IN1 — confirm physical board ID</t>
+          <t>M2S1371 / Switch 13-3 FB N | commissioned 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -28720,7 +28725,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>M2S1372 / Switch 13-3 FB R | ASSUMED on new C13-IN1 — confirm physical board ID</t>
+          <t>M2S1372 / Switch 13-3 FB R | commissioned 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -28755,7 +28760,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>ASSUMED on new C13-IN2 — confirm</t>
+          <t>local button; confirm silk</t>
         </is>
       </c>
     </row>
@@ -28790,7 +28795,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>ASSUMED on new C13-IN2 — confirm</t>
+          <t>local button; confirm silk</t>
         </is>
       </c>
     </row>
@@ -28825,7 +28830,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>ASSUMED on new C13-IN2 — confirm</t>
+          <t>local button; confirm silk</t>
         </is>
       </c>
     </row>
@@ -31565,9 +31570,39 @@
           <t>8LA</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>C13-OU3-1</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>C13-OU3-2</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>C13-OU3-3</t>
+        </is>
+      </c>
       <c r="P35" t="inlineStr">
         <is>
           <t>8LB / 8RB</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>C13-OU3-7</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>C13-OU3-8</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>C13-OU4-7</t>
         </is>
       </c>
     </row>

</xml_diff>